<commit_message>
fix: normalizar codigos BD jeans Dama PLANILLA 44 a 6 digitos
558 codigos convertidos: 4401->440100, 4414-00->441400, etc.
Esto hace que el VLOOKUP en TOMA DE PEDIDOS encuentre los articulos
en vez de retornar #N/D.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PLANILLA 44 LISTA PRECIO FINAL.xlsx
+++ b/PLANILLA 44 LISTA PRECIO FINAL.xlsx
@@ -23736,7 +23736,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr codeName="Hoja2">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -23782,7 +23782,7 @@
     <row r="2" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="223"/>
       <c r="B2" s="362">
-        <v>4401</v>
+        <v>440100</v>
       </c>
       <c r="C2" s="367"/>
       <c r="D2" s="358" t="s">
@@ -23796,7 +23796,7 @@
     <row r="3" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="223"/>
       <c r="B3" s="381">
-        <v>4402</v>
+        <v>440200</v>
       </c>
       <c r="C3" s="389" t="s">
         <v>522</v>
@@ -23814,7 +23814,7 @@
     <row r="4" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="223"/>
       <c r="B4" s="362">
-        <v>4403</v>
+        <v>440300</v>
       </c>
       <c r="C4" s="367"/>
       <c r="D4" s="358" t="s">
@@ -23828,7 +23828,7 @@
     <row r="5" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="223"/>
       <c r="B5" s="362">
-        <v>4404</v>
+        <v>440400</v>
       </c>
       <c r="C5" s="367"/>
       <c r="D5" s="358" t="s">
@@ -23842,7 +23842,7 @@
     <row r="6" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="223"/>
       <c r="B6" s="362">
-        <v>4405</v>
+        <v>440500</v>
       </c>
       <c r="C6" s="367"/>
       <c r="D6" s="358" t="s">
@@ -23856,7 +23856,7 @@
     <row r="7" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="223"/>
       <c r="B7" s="362">
-        <v>4406</v>
+        <v>440600</v>
       </c>
       <c r="C7" s="367" t="s">
         <v>524</v>
@@ -23874,7 +23874,7 @@
     <row r="8" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="223"/>
       <c r="B8" s="397">
-        <v>4407</v>
+        <v>440700</v>
       </c>
       <c r="C8" s="382" t="s">
         <v>525</v>
@@ -23892,7 +23892,7 @@
     <row r="9" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="223"/>
       <c r="B9" s="362">
-        <v>4408</v>
+        <v>440800</v>
       </c>
       <c r="C9" s="171"/>
       <c r="D9" s="358" t="s">
@@ -23906,7 +23906,7 @@
     <row r="10" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="224"/>
       <c r="B10" s="362">
-        <v>4409</v>
+        <v>440900</v>
       </c>
       <c r="C10" s="171"/>
       <c r="D10" s="358" t="s">
@@ -23920,7 +23920,7 @@
     <row r="11" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="224"/>
       <c r="B11" s="362">
-        <v>4410</v>
+        <v>441000</v>
       </c>
       <c r="C11" s="171"/>
       <c r="D11" s="358" t="s">
@@ -23934,7 +23934,7 @@
     <row r="12" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="223"/>
       <c r="B12" s="362">
-        <v>4411</v>
+        <v>441100</v>
       </c>
       <c r="C12" s="171"/>
       <c r="D12" s="358" t="s">
@@ -23948,7 +23948,7 @@
     <row r="13" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="223"/>
       <c r="B13" s="397">
-        <v>4412</v>
+        <v>441200</v>
       </c>
       <c r="C13" s="382" t="s">
         <v>526</v>
@@ -23966,7 +23966,7 @@
     <row r="14" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="223"/>
       <c r="B14" s="381">
-        <v>4413</v>
+        <v>441300</v>
       </c>
       <c r="C14" s="382" t="s">
         <v>528</v>
@@ -23983,8 +23983,8 @@
     </row>
     <row r="15" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="223"/>
-      <c r="B15" s="381" t="s">
-        <v>2219</v>
+      <c r="B15" s="381">
+        <v>441400</v>
       </c>
       <c r="C15" s="382" t="s">
         <v>529</v>
@@ -24001,8 +24001,8 @@
     </row>
     <row r="16" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="223"/>
-      <c r="B16" s="381" t="s">
-        <v>530</v>
+      <c r="B16" s="381">
+        <v>441401</v>
       </c>
       <c r="C16" s="382" t="s">
         <v>531</v>
@@ -24019,8 +24019,8 @@
     </row>
     <row r="17" spans="1:11" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="223"/>
-      <c r="B17" s="362" t="s">
-        <v>2214</v>
+      <c r="B17" s="362">
+        <v>441500</v>
       </c>
       <c r="C17" s="171" t="s">
         <v>2212</v>
@@ -24033,8 +24033,8 @@
     </row>
     <row r="18" spans="1:11" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="223"/>
-      <c r="B18" s="362" t="s">
-        <v>2213</v>
+      <c r="B18" s="362">
+        <v>441501</v>
       </c>
       <c r="C18" s="171" t="s">
         <v>2211</v>
@@ -24048,7 +24048,7 @@
     <row r="19" spans="1:11" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="223"/>
       <c r="B19" s="397">
-        <v>4416</v>
+        <v>441600</v>
       </c>
       <c r="C19" s="382" t="s">
         <v>532</v>
@@ -24102,7 +24102,7 @@
     <row r="22" spans="1:11" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="223"/>
       <c r="B22" s="397">
-        <v>4418</v>
+        <v>441800</v>
       </c>
       <c r="C22" s="382" t="s">
         <v>534</v>
@@ -24119,8 +24119,8 @@
     </row>
     <row r="23" spans="1:11" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="223"/>
-      <c r="B23" s="397" t="s">
-        <v>535</v>
+      <c r="B23" s="397">
+        <v>441900</v>
       </c>
       <c r="C23" s="382" t="s">
         <v>536</v>
@@ -24137,8 +24137,8 @@
     </row>
     <row r="24" spans="1:11" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="223"/>
-      <c r="B24" s="397" t="s">
-        <v>537</v>
+      <c r="B24" s="397">
+        <v>441901</v>
       </c>
       <c r="C24" s="382" t="s">
         <v>538</v>
@@ -24156,7 +24156,7 @@
     <row r="25" spans="1:11" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="223"/>
       <c r="B25" s="362">
-        <v>4420</v>
+        <v>442000</v>
       </c>
       <c r="C25" s="378" t="s">
         <v>539</v>
@@ -24171,8 +24171,8 @@
     </row>
     <row r="26" spans="1:11" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="223"/>
-      <c r="B26" s="397" t="s">
-        <v>2223</v>
+      <c r="B26" s="397">
+        <v>442100</v>
       </c>
       <c r="C26" s="382" t="s">
         <v>2225</v>
@@ -24193,8 +24193,8 @@
     </row>
     <row r="27" spans="1:11" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="223"/>
-      <c r="B27" s="397" t="s">
-        <v>2224</v>
+      <c r="B27" s="397">
+        <v>442101</v>
       </c>
       <c r="C27" s="382" t="s">
         <v>2226</v>
@@ -24211,8 +24211,8 @@
     </row>
     <row r="28" spans="1:11" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="223"/>
-      <c r="B28" s="381" t="s">
-        <v>541</v>
+      <c r="B28" s="381">
+        <v>442200</v>
       </c>
       <c r="C28" s="382" t="s">
         <v>542</v>
@@ -24229,8 +24229,8 @@
     </row>
     <row r="29" spans="1:11" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="223"/>
-      <c r="B29" s="381" t="s">
-        <v>544</v>
+      <c r="B29" s="381">
+        <v>442204</v>
       </c>
       <c r="C29" s="382" t="s">
         <v>545</v>
@@ -24247,8 +24247,8 @@
     </row>
     <row r="30" spans="1:11" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="223"/>
-      <c r="B30" s="381" t="s">
-        <v>546</v>
+      <c r="B30" s="381">
+        <v>442206</v>
       </c>
       <c r="C30" s="382" t="s">
         <v>547</v>
@@ -24265,8 +24265,8 @@
     </row>
     <row r="31" spans="1:11" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="223"/>
-      <c r="B31" s="381" t="s">
-        <v>548</v>
+      <c r="B31" s="381">
+        <v>442238</v>
       </c>
       <c r="C31" s="382" t="s">
         <v>549</v>
@@ -24284,7 +24284,7 @@
     <row r="32" spans="1:11" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="223"/>
       <c r="B32" s="362">
-        <v>4423</v>
+        <v>442300</v>
       </c>
       <c r="C32" s="171"/>
       <c r="D32" s="358" t="s">
@@ -24298,7 +24298,7 @@
     <row r="33" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="223"/>
       <c r="B33" s="362">
-        <v>4424</v>
+        <v>442400</v>
       </c>
       <c r="C33" s="171"/>
       <c r="D33" s="358" t="s">
@@ -24312,7 +24312,7 @@
     <row r="34" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="223"/>
       <c r="B34" s="362">
-        <v>4425</v>
+        <v>442500</v>
       </c>
       <c r="C34" s="171"/>
       <c r="D34" s="358" t="s">
@@ -24325,8 +24325,8 @@
     </row>
     <row r="35" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="223"/>
-      <c r="B35" s="381" t="s">
-        <v>2216</v>
+      <c r="B35" s="381">
+        <v>442600</v>
       </c>
       <c r="C35" s="393" t="s">
         <v>551</v>
@@ -24343,8 +24343,8 @@
     </row>
     <row r="36" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="223"/>
-      <c r="B36" s="381" t="s">
-        <v>2217</v>
+      <c r="B36" s="381">
+        <v>442601</v>
       </c>
       <c r="C36" s="393" t="s">
         <v>2218</v>
@@ -24362,7 +24362,7 @@
     <row r="37" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="225"/>
       <c r="B37" s="362">
-        <v>4427</v>
+        <v>442700</v>
       </c>
       <c r="C37" s="171"/>
       <c r="D37" s="358" t="s">
@@ -24376,7 +24376,7 @@
     <row r="38" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="225"/>
       <c r="B38" s="362">
-        <v>4428</v>
+        <v>442800</v>
       </c>
       <c r="C38" s="171"/>
       <c r="D38" s="358" t="s">
@@ -24389,8 +24389,8 @@
     </row>
     <row r="39" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="224"/>
-      <c r="B39" s="362" t="s">
-        <v>2193</v>
+      <c r="B39" s="362">
+        <v>442909</v>
       </c>
       <c r="C39" s="171" t="s">
         <v>2194</v>
@@ -24407,8 +24407,8 @@
     </row>
     <row r="40" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="226"/>
-      <c r="B40" s="362" t="s">
-        <v>2195</v>
+      <c r="B40" s="362">
+        <v>442904</v>
       </c>
       <c r="C40" s="171" t="s">
         <v>2196</v>
@@ -24425,8 +24425,8 @@
     </row>
     <row r="41" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="224"/>
-      <c r="B41" s="362" t="s">
-        <v>2197</v>
+      <c r="B41" s="362">
+        <v>442906</v>
       </c>
       <c r="C41" s="171" t="s">
         <v>2198</v>
@@ -24443,8 +24443,8 @@
     </row>
     <row r="42" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="224"/>
-      <c r="B42" s="362" t="s">
-        <v>2199</v>
+      <c r="B42" s="362">
+        <v>442924</v>
       </c>
       <c r="C42" s="171" t="s">
         <v>2200</v>
@@ -24461,8 +24461,8 @@
     </row>
     <row r="43" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="224"/>
-      <c r="B43" s="362" t="s">
-        <v>2201</v>
+      <c r="B43" s="362">
+        <v>442938</v>
       </c>
       <c r="C43" s="171" t="s">
         <v>2202</v>
@@ -24488,7 +24488,7 @@
     <row r="45" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="224"/>
       <c r="B45" s="397">
-        <v>4430</v>
+        <v>443000</v>
       </c>
       <c r="C45" s="171" t="s">
         <v>552</v>
@@ -24505,8 +24505,8 @@
     </row>
     <row r="46" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="224"/>
-      <c r="B46" s="397" t="s">
-        <v>553</v>
+      <c r="B46" s="397">
+        <v>443100</v>
       </c>
       <c r="C46" s="382" t="s">
         <v>554</v>
@@ -24523,8 +24523,8 @@
     </row>
     <row r="47" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="224"/>
-      <c r="B47" s="397" t="s">
-        <v>555</v>
+      <c r="B47" s="397">
+        <v>443101</v>
       </c>
       <c r="C47" s="386" t="s">
         <v>556</v>
@@ -24542,7 +24542,7 @@
     <row r="48" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="224"/>
       <c r="B48" s="381">
-        <v>4432</v>
+        <v>443200</v>
       </c>
       <c r="C48" s="382" t="s">
         <v>557</v>
@@ -24560,7 +24560,7 @@
     <row r="49" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="224"/>
       <c r="B49" s="362">
-        <v>4433</v>
+        <v>443300</v>
       </c>
       <c r="C49" s="171" t="s">
         <v>558</v>
@@ -24576,7 +24576,7 @@
     <row r="50" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="224"/>
       <c r="B50" s="397">
-        <v>4434</v>
+        <v>443400</v>
       </c>
       <c r="C50" s="386" t="s">
         <v>560</v>
@@ -24594,7 +24594,7 @@
     <row r="51" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="224"/>
       <c r="B51" s="381">
-        <v>4435</v>
+        <v>443500</v>
       </c>
       <c r="C51" s="393" t="s">
         <v>561</v>
@@ -24612,7 +24612,7 @@
     <row r="52" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="224"/>
       <c r="B52" s="362">
-        <v>4436</v>
+        <v>443600</v>
       </c>
       <c r="C52" s="171"/>
       <c r="D52" s="358" t="s">
@@ -24626,7 +24626,7 @@
     <row r="53" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="227"/>
       <c r="B53" s="362">
-        <v>4437</v>
+        <v>443700</v>
       </c>
       <c r="C53" s="171" t="s">
         <v>562</v>
@@ -24642,7 +24642,7 @@
     <row r="54" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="227"/>
       <c r="B54" s="362">
-        <v>4438</v>
+        <v>443800</v>
       </c>
       <c r="C54" s="171" t="s">
         <v>2215</v>
@@ -24655,8 +24655,8 @@
     </row>
     <row r="55" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="228"/>
-      <c r="B55" s="362" t="s">
-        <v>563</v>
+      <c r="B55" s="362">
+        <v>443900</v>
       </c>
       <c r="C55" s="171" t="s">
         <v>564</v>
@@ -24672,7 +24672,7 @@
     <row r="56" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="228"/>
       <c r="B56" s="381">
-        <v>4440</v>
+        <v>444000</v>
       </c>
       <c r="C56" s="382" t="s">
         <v>565</v>
@@ -24690,7 +24690,7 @@
     <row r="57" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="224"/>
       <c r="B57" s="397">
-        <v>4441</v>
+        <v>444100</v>
       </c>
       <c r="C57" s="394" t="s">
         <v>566</v>
@@ -24708,7 +24708,7 @@
     <row r="58" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="224"/>
       <c r="B58" s="381">
-        <v>4442</v>
+        <v>444200</v>
       </c>
       <c r="C58" s="382" t="s">
         <v>567</v>
@@ -24726,7 +24726,7 @@
     <row r="59" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="224"/>
       <c r="B59" s="381">
-        <v>4443</v>
+        <v>444300</v>
       </c>
       <c r="C59" s="382" t="s">
         <v>569</v>
@@ -24744,7 +24744,7 @@
     <row r="60" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="224"/>
       <c r="B60" s="381">
-        <v>4444</v>
+        <v>444400</v>
       </c>
       <c r="C60" s="382" t="s">
         <v>570</v>
@@ -24762,7 +24762,7 @@
     <row r="61" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="224"/>
       <c r="B61" s="362">
-        <v>4445</v>
+        <v>444500</v>
       </c>
       <c r="C61" s="171"/>
       <c r="D61" s="358" t="s">
@@ -24776,7 +24776,7 @@
     <row r="62" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="224"/>
       <c r="B62" s="362">
-        <v>4446</v>
+        <v>444600</v>
       </c>
       <c r="C62" s="171"/>
       <c r="D62" s="358" t="s">
@@ -24790,7 +24790,7 @@
     <row r="63" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="224"/>
       <c r="B63" s="362">
-        <v>4447</v>
+        <v>444700</v>
       </c>
       <c r="C63" s="171"/>
       <c r="D63" s="358" t="s">
@@ -24804,7 +24804,7 @@
     <row r="64" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="224"/>
       <c r="B64" s="381">
-        <v>4448</v>
+        <v>444800</v>
       </c>
       <c r="C64" s="382" t="s">
         <v>571</v>
@@ -24821,8 +24821,8 @@
     </row>
     <row r="65" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="224"/>
-      <c r="B65" s="362" t="s">
-        <v>572</v>
+      <c r="B65" s="362">
+        <v>444890</v>
       </c>
       <c r="C65" s="378" t="s">
         <v>573</v>
@@ -24836,7 +24836,7 @@
     <row r="66" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="224"/>
       <c r="B66" s="362">
-        <v>4449</v>
+        <v>444900</v>
       </c>
       <c r="C66" s="171"/>
       <c r="D66" s="358" t="s">
@@ -24850,7 +24850,7 @@
     <row r="67" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="224"/>
       <c r="B67" s="362">
-        <v>4450</v>
+        <v>445000</v>
       </c>
       <c r="C67" s="171"/>
       <c r="D67" s="358" t="s">
@@ -24864,7 +24864,7 @@
     <row r="68" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="224"/>
       <c r="B68" s="362">
-        <v>4451</v>
+        <v>445100</v>
       </c>
       <c r="C68" s="171"/>
       <c r="D68" s="361" t="s">
@@ -24878,7 +24878,7 @@
     <row r="69" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="224"/>
       <c r="B69" s="362">
-        <v>4452</v>
+        <v>445200</v>
       </c>
       <c r="C69" s="171"/>
       <c r="D69" s="358" t="s">
@@ -24892,7 +24892,7 @@
     <row r="70" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="224"/>
       <c r="B70" s="381">
-        <v>4453</v>
+        <v>445300</v>
       </c>
       <c r="C70" s="382" t="s">
         <v>574</v>
@@ -24910,7 +24910,7 @@
     <row r="71" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="224"/>
       <c r="B71" s="397">
-        <v>4454</v>
+        <v>445400</v>
       </c>
       <c r="C71" s="382" t="s">
         <v>576</v>
@@ -24928,7 +24928,7 @@
     <row r="72" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="224"/>
       <c r="B72" s="397">
-        <v>4455</v>
+        <v>445500</v>
       </c>
       <c r="C72" s="382" t="s">
         <v>577</v>
@@ -24945,8 +24945,8 @@
     </row>
     <row r="73" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="224"/>
-      <c r="B73" s="381" t="s">
-        <v>2220</v>
+      <c r="B73" s="381">
+        <v>445660</v>
       </c>
       <c r="C73" s="386" t="s">
         <v>2222</v>
@@ -24963,8 +24963,8 @@
     </row>
     <row r="74" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="224"/>
-      <c r="B74" s="381" t="s">
-        <v>2221</v>
+      <c r="B74" s="381">
+        <v>445600</v>
       </c>
       <c r="C74" s="386" t="s">
         <v>2222</v>
@@ -24981,8 +24981,8 @@
     </row>
     <row r="75" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="224"/>
-      <c r="B75" s="381" t="s">
-        <v>578</v>
+      <c r="B75" s="381">
+        <v>445700</v>
       </c>
       <c r="C75" s="382" t="s">
         <v>579</v>
@@ -24999,8 +24999,8 @@
     </row>
     <row r="76" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="224"/>
-      <c r="B76" s="381" t="s">
-        <v>580</v>
+      <c r="B76" s="381">
+        <v>445738</v>
       </c>
       <c r="C76" s="382" t="s">
         <v>581</v>
@@ -25017,8 +25017,8 @@
     </row>
     <row r="77" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="224"/>
-      <c r="B77" s="381" t="s">
-        <v>582</v>
+      <c r="B77" s="381">
+        <v>445706</v>
       </c>
       <c r="C77" s="382" t="s">
         <v>583</v>
@@ -25035,8 +25035,8 @@
     </row>
     <row r="78" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="224"/>
-      <c r="B78" s="381" t="s">
-        <v>584</v>
+      <c r="B78" s="381">
+        <v>445704</v>
       </c>
       <c r="C78" s="382" t="s">
         <v>585</v>
@@ -25053,8 +25053,8 @@
     </row>
     <row r="79" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="224"/>
-      <c r="B79" s="381" t="s">
-        <v>2203</v>
+      <c r="B79" s="381">
+        <v>445724</v>
       </c>
       <c r="C79" s="382" t="s">
         <v>2204</v>
@@ -25072,7 +25072,7 @@
     <row r="80" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="224"/>
       <c r="B80" s="381">
-        <v>4458</v>
+        <v>445800</v>
       </c>
       <c r="C80" s="382" t="s">
         <v>586</v>
@@ -25110,7 +25110,7 @@
         <v>16</v>
       </c>
       <c r="B83" s="362">
-        <v>4458</v>
+        <v>445800</v>
       </c>
       <c r="C83" s="171" t="s">
         <v>588</v>
@@ -25130,7 +25130,7 @@
         <v>17</v>
       </c>
       <c r="B84" s="381">
-        <v>4459</v>
+        <v>445900</v>
       </c>
       <c r="C84" s="382" t="s">
         <v>589</v>
@@ -25150,7 +25150,7 @@
         <v>18</v>
       </c>
       <c r="B85" s="362">
-        <v>4460</v>
+        <v>446000</v>
       </c>
       <c r="C85" s="171" t="s">
         <v>591</v>
@@ -25170,7 +25170,7 @@
         <v>19</v>
       </c>
       <c r="B86" s="362">
-        <v>4461</v>
+        <v>446100</v>
       </c>
       <c r="C86" s="171"/>
       <c r="D86" s="358" t="s">
@@ -25186,7 +25186,7 @@
         <v>20</v>
       </c>
       <c r="B87" s="362">
-        <v>4462</v>
+        <v>446200</v>
       </c>
       <c r="C87" s="171"/>
       <c r="D87" s="358" t="s">
@@ -25202,7 +25202,7 @@
         <v>3955</v>
       </c>
       <c r="B88" s="362">
-        <v>4463</v>
+        <v>446300</v>
       </c>
       <c r="C88" s="171"/>
       <c r="D88" s="358" t="s">
@@ -25218,7 +25218,7 @@
         <v>3957</v>
       </c>
       <c r="B89" s="362">
-        <v>4464</v>
+        <v>446400</v>
       </c>
       <c r="C89" s="171"/>
       <c r="D89" s="358" t="s">
@@ -25234,7 +25234,7 @@
         <v>21</v>
       </c>
       <c r="B90" s="362">
-        <v>4465</v>
+        <v>446500</v>
       </c>
       <c r="C90" s="171"/>
       <c r="D90" s="358" t="s">
@@ -25250,7 +25250,7 @@
         <v>22</v>
       </c>
       <c r="B91" s="362">
-        <v>4466</v>
+        <v>446600</v>
       </c>
       <c r="C91" s="171"/>
       <c r="D91" s="358" t="s">
@@ -25266,7 +25266,7 @@
         <v>23</v>
       </c>
       <c r="B92" s="362">
-        <v>4467</v>
+        <v>446700</v>
       </c>
       <c r="C92" s="171"/>
       <c r="D92" s="358" t="s">
@@ -25282,7 +25282,7 @@
         <v>24</v>
       </c>
       <c r="B93" s="397">
-        <v>4468</v>
+        <v>446800</v>
       </c>
       <c r="C93" s="382" t="s">
         <v>593</v>
@@ -25302,7 +25302,7 @@
         <v>3961</v>
       </c>
       <c r="B94" s="362">
-        <v>4469</v>
+        <v>446900</v>
       </c>
       <c r="C94" s="171"/>
       <c r="D94" s="358" t="s">
@@ -25320,7 +25320,7 @@
         <v>3962</v>
       </c>
       <c r="B95" s="362">
-        <v>4470</v>
+        <v>447000</v>
       </c>
       <c r="C95" s="171"/>
       <c r="D95" s="358" t="s">
@@ -25338,7 +25338,7 @@
         <v>25</v>
       </c>
       <c r="B96" s="397">
-        <v>4471</v>
+        <v>447100</v>
       </c>
       <c r="C96" s="382" t="s">
         <v>596</v>
@@ -25357,8 +25357,8 @@
       <c r="A97" s="224">
         <v>3967</v>
       </c>
-      <c r="B97" s="397" t="s">
-        <v>597</v>
+      <c r="B97" s="397">
+        <v>447200</v>
       </c>
       <c r="C97" s="386" t="s">
         <v>598</v>
@@ -25377,8 +25377,8 @@
       <c r="A98" s="224">
         <v>3968</v>
       </c>
-      <c r="B98" s="397" t="s">
-        <v>599</v>
+      <c r="B98" s="397">
+        <v>447201</v>
       </c>
       <c r="C98" s="386" t="s">
         <v>600</v>
@@ -25398,7 +25398,7 @@
         <v>26</v>
       </c>
       <c r="B99" s="397">
-        <v>4473</v>
+        <v>447300</v>
       </c>
       <c r="C99" s="382" t="s">
         <v>602</v>
@@ -25418,7 +25418,7 @@
         <v>27</v>
       </c>
       <c r="B100" s="362">
-        <v>4474</v>
+        <v>447400</v>
       </c>
       <c r="C100" s="171"/>
       <c r="D100" s="363" t="s">
@@ -25434,7 +25434,7 @@
         <v>28</v>
       </c>
       <c r="B101" s="362">
-        <v>4475</v>
+        <v>447500</v>
       </c>
       <c r="C101" s="171"/>
       <c r="D101" s="362"/>
@@ -25446,7 +25446,7 @@
         <v>29</v>
       </c>
       <c r="B102" s="397">
-        <v>4476</v>
+        <v>447600</v>
       </c>
       <c r="C102" s="171" t="s">
         <v>2180</v>
@@ -25466,7 +25466,7 @@
         <v>30</v>
       </c>
       <c r="B103" s="380">
-        <v>4477</v>
+        <v>447700</v>
       </c>
       <c r="C103" s="171"/>
       <c r="D103" s="170"/>
@@ -25478,7 +25478,7 @@
         <v>3972</v>
       </c>
       <c r="B104" s="380">
-        <v>4478</v>
+        <v>447800</v>
       </c>
       <c r="C104" s="171"/>
       <c r="D104" s="170"/>
@@ -25490,7 +25490,7 @@
         <v>3984</v>
       </c>
       <c r="B105" s="362">
-        <v>4479</v>
+        <v>447900</v>
       </c>
       <c r="C105" s="171"/>
       <c r="D105" s="170"/>
@@ -25502,7 +25502,7 @@
         <v>3985</v>
       </c>
       <c r="B106" s="396">
-        <v>4480</v>
+        <v>448000</v>
       </c>
       <c r="C106" s="395" t="s">
         <v>2191</v>
@@ -25522,7 +25522,7 @@
         <v>3990</v>
       </c>
       <c r="B107" s="380">
-        <v>4481</v>
+        <v>448100</v>
       </c>
       <c r="C107" s="171"/>
       <c r="D107" s="170"/>
@@ -25534,7 +25534,7 @@
         <v>4001</v>
       </c>
       <c r="B108" s="397">
-        <v>4482</v>
+        <v>448200</v>
       </c>
       <c r="C108" s="171" t="s">
         <v>2189</v>
@@ -25566,7 +25566,7 @@
         <v>4003</v>
       </c>
       <c r="B109" s="380">
-        <v>4483</v>
+        <v>448300</v>
       </c>
       <c r="C109" s="171"/>
       <c r="D109" s="170"/>
@@ -25591,7 +25591,7 @@
         <v>4008</v>
       </c>
       <c r="B110" s="396">
-        <v>4484</v>
+        <v>448400</v>
       </c>
       <c r="C110" s="171" t="s">
         <v>2182</v>
@@ -25624,7 +25624,7 @@
         <v>4009</v>
       </c>
       <c r="B111" s="397">
-        <v>4485</v>
+        <v>448500</v>
       </c>
       <c r="C111" s="171" t="s">
         <v>2181</v>
@@ -25656,7 +25656,7 @@
         <v>4010</v>
       </c>
       <c r="B112" s="396">
-        <v>4486</v>
+        <v>448600</v>
       </c>
       <c r="C112" s="171" t="s">
         <v>2187</v>
@@ -25687,8 +25687,8 @@
       <c r="A113" s="230">
         <v>4013</v>
       </c>
-      <c r="B113" s="380" t="s">
-        <v>2183</v>
+      <c r="B113" s="380">
+        <v>448760</v>
       </c>
       <c r="C113" s="171" t="s">
         <v>2185</v>
@@ -25720,7 +25720,7 @@
         <v>4018</v>
       </c>
       <c r="B114" s="380">
-        <v>4487</v>
+        <v>448700</v>
       </c>
       <c r="C114" s="171" t="s">
         <v>2184</v>
@@ -25752,7 +25752,7 @@
         <v>4019</v>
       </c>
       <c r="B115" s="362">
-        <v>4488</v>
+        <v>448800</v>
       </c>
       <c r="C115" s="171" t="s">
         <v>605</v>
@@ -25784,7 +25784,7 @@
         <v>4019</v>
       </c>
       <c r="B116" s="396">
-        <v>4489</v>
+        <v>448900</v>
       </c>
       <c r="C116" s="382" t="s">
         <v>606</v>
@@ -25816,7 +25816,7 @@
         <v>4024</v>
       </c>
       <c r="B117" s="380">
-        <v>4490</v>
+        <v>449000</v>
       </c>
       <c r="C117" s="171"/>
       <c r="D117" s="170"/>
@@ -25832,7 +25832,7 @@
         <v>4026</v>
       </c>
       <c r="B118" s="362">
-        <v>4491</v>
+        <v>449100</v>
       </c>
       <c r="C118" s="171"/>
       <c r="D118" s="170"/>
@@ -25855,8 +25855,8 @@
       <c r="A119" s="232">
         <v>4028</v>
       </c>
-      <c r="B119" s="396" t="s">
-        <v>607</v>
+      <c r="B119" s="396">
+        <v>449200</v>
       </c>
       <c r="C119" s="171" t="s">
         <v>608</v>
@@ -25887,8 +25887,8 @@
       <c r="A120" s="232">
         <v>4033</v>
       </c>
-      <c r="B120" s="380" t="s">
-        <v>609</v>
+      <c r="B120" s="380">
+        <v>449290</v>
       </c>
       <c r="C120" s="171" t="s">
         <v>610</v>
@@ -25919,8 +25919,8 @@
       <c r="A121" s="233">
         <v>4034</v>
       </c>
-      <c r="B121" s="380" t="s">
-        <v>2209</v>
+      <c r="B121" s="380">
+        <v>449301</v>
       </c>
       <c r="C121" s="171" t="s">
         <v>2210</v>
@@ -25943,8 +25943,8 @@
       <c r="A122" s="230">
         <v>4035</v>
       </c>
-      <c r="B122" s="397" t="s">
-        <v>611</v>
+      <c r="B122" s="397">
+        <v>449404</v>
       </c>
       <c r="C122" s="171" t="s">
         <v>2205</v>
@@ -25975,8 +25975,8 @@
       <c r="A123" s="230">
         <v>4036</v>
       </c>
-      <c r="B123" s="362" t="s">
-        <v>612</v>
+      <c r="B123" s="362">
+        <v>449406</v>
       </c>
       <c r="C123" s="171" t="s">
         <v>2206</v>
@@ -26007,8 +26007,8 @@
       <c r="A124" s="234">
         <v>4042</v>
       </c>
-      <c r="B124" s="362" t="s">
-        <v>613</v>
+      <c r="B124" s="362">
+        <v>449409</v>
       </c>
       <c r="C124" s="171" t="s">
         <v>2207</v>
@@ -26039,8 +26039,8 @@
       <c r="A125" s="235">
         <v>4044</v>
       </c>
-      <c r="B125" s="362" t="s">
-        <v>614</v>
+      <c r="B125" s="362">
+        <v>449424</v>
       </c>
       <c r="C125" s="171" t="s">
         <v>2208</v>
@@ -26107,8 +26107,8 @@
       <c r="A128" s="236">
         <v>4051</v>
       </c>
-      <c r="B128" s="380" t="s">
-        <v>615</v>
+      <c r="B128" s="380">
+        <v>449500</v>
       </c>
       <c r="C128" s="171" t="s">
         <v>616</v>
@@ -26139,8 +26139,8 @@
       <c r="A129" s="236">
         <v>4052</v>
       </c>
-      <c r="B129" s="380" t="s">
-        <v>617</v>
+      <c r="B129" s="380">
+        <v>449504</v>
       </c>
       <c r="C129" s="171" t="s">
         <v>618</v>
@@ -26171,8 +26171,8 @@
       <c r="A130" s="237">
         <v>4053</v>
       </c>
-      <c r="B130" s="380" t="s">
-        <v>619</v>
+      <c r="B130" s="380">
+        <v>449506</v>
       </c>
       <c r="C130" s="171" t="s">
         <v>620</v>
@@ -26203,8 +26203,8 @@
       <c r="A131" s="238">
         <v>4053</v>
       </c>
-      <c r="B131" s="380" t="s">
-        <v>621</v>
+      <c r="B131" s="380">
+        <v>449509</v>
       </c>
       <c r="C131" s="171" t="s">
         <v>622</v>
@@ -26227,8 +26227,8 @@
       <c r="A132" s="239">
         <v>4056</v>
       </c>
-      <c r="B132" s="380" t="s">
-        <v>623</v>
+      <c r="B132" s="380">
+        <v>449524</v>
       </c>
       <c r="C132" s="171" t="s">
         <v>624</v>
@@ -26259,8 +26259,8 @@
       <c r="A133" s="216">
         <v>4060</v>
       </c>
-      <c r="B133" s="380" t="s">
-        <v>625</v>
+      <c r="B133" s="380">
+        <v>449538</v>
       </c>
       <c r="C133" s="171" t="s">
         <v>626</v>
@@ -26292,7 +26292,7 @@
         <v>4061</v>
       </c>
       <c r="B134" s="391">
-        <v>4496</v>
+        <v>449600</v>
       </c>
       <c r="C134" s="382" t="s">
         <v>2192</v>
@@ -26324,7 +26324,7 @@
         <v>4061</v>
       </c>
       <c r="B135" s="397">
-        <v>4497</v>
+        <v>449700</v>
       </c>
       <c r="C135" s="171" t="s">
         <v>2190</v>
@@ -26348,7 +26348,7 @@
         <v>4064</v>
       </c>
       <c r="B136" s="380">
-        <v>4498</v>
+        <v>449800</v>
       </c>
       <c r="C136" s="171"/>
       <c r="D136" s="170"/>
@@ -26372,7 +26372,7 @@
         <v>4065</v>
       </c>
       <c r="B137" s="295">
-        <v>4499</v>
+        <v>449900</v>
       </c>
       <c r="F137" s="380"/>
       <c r="I137" s="157">
@@ -26393,7 +26393,7 @@
         <v>4065</v>
       </c>
       <c r="B138" s="215">
-        <v>4065</v>
+        <v>406500</v>
       </c>
       <c r="C138" s="171" t="s">
         <v>40</v>
@@ -26425,7 +26425,7 @@
         <v>4076</v>
       </c>
       <c r="B139" s="215">
-        <v>4076</v>
+        <v>407600</v>
       </c>
       <c r="C139" s="171" t="s">
         <v>42</v>
@@ -26456,8 +26456,8 @@
       <c r="A140" s="241" t="s">
         <v>38</v>
       </c>
-      <c r="B140" s="241" t="s">
-        <v>38</v>
+      <c r="B140" s="241">
+        <v>400200</v>
       </c>
       <c r="C140" s="171" t="s">
         <v>43</v>
@@ -26488,8 +26488,8 @@
       <c r="A141" s="241" t="s">
         <v>38</v>
       </c>
-      <c r="B141" s="241" t="s">
-        <v>38</v>
+      <c r="B141" s="241">
+        <v>400200</v>
       </c>
       <c r="C141" s="171"/>
       <c r="D141" s="177" t="s">
@@ -26518,8 +26518,8 @@
       <c r="A142" s="215" t="s">
         <v>38</v>
       </c>
-      <c r="B142" s="215" t="s">
-        <v>38</v>
+      <c r="B142" s="215">
+        <v>400200</v>
       </c>
       <c r="C142" s="171" t="s">
         <v>44</v>
@@ -26550,8 +26550,8 @@
       <c r="A143" s="241" t="s">
         <v>45</v>
       </c>
-      <c r="B143" s="241" t="s">
-        <v>45</v>
+      <c r="B143" s="241">
+        <v>400201</v>
       </c>
       <c r="C143" s="171" t="s">
         <v>46</v>
@@ -26582,8 +26582,8 @@
       <c r="A144" s="215" t="s">
         <v>45</v>
       </c>
-      <c r="B144" s="215" t="s">
-        <v>45</v>
+      <c r="B144" s="215">
+        <v>400201</v>
       </c>
       <c r="C144" s="171" t="s">
         <v>47</v>
@@ -26606,8 +26606,8 @@
       <c r="A145" s="241" t="s">
         <v>39</v>
       </c>
-      <c r="B145" s="241" t="s">
-        <v>39</v>
+      <c r="B145" s="241">
+        <v>400203</v>
       </c>
       <c r="C145" s="171"/>
       <c r="D145" s="177" t="s">
@@ -26636,8 +26636,8 @@
       <c r="A146" s="241" t="s">
         <v>49</v>
       </c>
-      <c r="B146" s="241" t="s">
-        <v>49</v>
+      <c r="B146" s="241">
+        <v>400400</v>
       </c>
       <c r="C146" s="171" t="s">
         <v>50</v>
@@ -26668,8 +26668,8 @@
       <c r="A147" s="215" t="s">
         <v>49</v>
       </c>
-      <c r="B147" s="215" t="s">
-        <v>49</v>
+      <c r="B147" s="215">
+        <v>400400</v>
       </c>
       <c r="C147" s="171" t="s">
         <v>51</v>
@@ -26692,8 +26692,8 @@
       <c r="A148" s="241" t="s">
         <v>52</v>
       </c>
-      <c r="B148" s="241" t="s">
-        <v>52</v>
+      <c r="B148" s="241">
+        <v>400401</v>
       </c>
       <c r="C148" s="171" t="s">
         <v>53</v>
@@ -26724,8 +26724,8 @@
       <c r="A149" s="215" t="s">
         <v>52</v>
       </c>
-      <c r="B149" s="215" t="s">
-        <v>52</v>
+      <c r="B149" s="215">
+        <v>400401</v>
       </c>
       <c r="C149" s="171" t="s">
         <v>54</v>
@@ -26756,8 +26756,8 @@
       <c r="A150" s="241" t="s">
         <v>56</v>
       </c>
-      <c r="B150" s="241" t="s">
-        <v>56</v>
+      <c r="B150" s="241">
+        <v>400700</v>
       </c>
       <c r="C150" s="171" t="s">
         <v>57</v>
@@ -26788,8 +26788,8 @@
       <c r="A151" s="215" t="s">
         <v>48</v>
       </c>
-      <c r="B151" s="215" t="s">
-        <v>48</v>
+      <c r="B151" s="215">
+        <v>400790</v>
       </c>
       <c r="C151" s="171" t="s">
         <v>58</v>
@@ -26820,8 +26820,8 @@
       <c r="A152" s="241" t="s">
         <v>48</v>
       </c>
-      <c r="B152" s="241" t="s">
-        <v>48</v>
+      <c r="B152" s="241">
+        <v>400790</v>
       </c>
       <c r="C152" s="171"/>
       <c r="D152" s="177" t="s">
@@ -26850,8 +26850,8 @@
       <c r="A153" s="215" t="s">
         <v>48</v>
       </c>
-      <c r="B153" s="215" t="s">
-        <v>48</v>
+      <c r="B153" s="215">
+        <v>400790</v>
       </c>
       <c r="C153" s="171" t="s">
         <v>58</v>
@@ -26882,8 +26882,8 @@
       <c r="A154" s="241" t="s">
         <v>59</v>
       </c>
-      <c r="B154" s="241" t="s">
-        <v>59</v>
+      <c r="B154" s="241">
+        <v>401100</v>
       </c>
       <c r="C154" s="171" t="s">
         <v>60</v>
@@ -26914,8 +26914,8 @@
       <c r="A155" s="241" t="s">
         <v>61</v>
       </c>
-      <c r="B155" s="241" t="s">
-        <v>61</v>
+      <c r="B155" s="241">
+        <v>401101</v>
       </c>
       <c r="C155" s="171" t="s">
         <v>62</v>
@@ -26946,8 +26946,8 @@
       <c r="A156" s="241" t="s">
         <v>64</v>
       </c>
-      <c r="B156" s="241" t="s">
-        <v>64</v>
+      <c r="B156" s="241">
+        <v>401101</v>
       </c>
       <c r="C156" s="171" t="s">
         <v>65</v>
@@ -26978,8 +26978,8 @@
       <c r="A157" s="242" t="s">
         <v>67</v>
       </c>
-      <c r="B157" s="242" t="s">
-        <v>67</v>
+      <c r="B157" s="242">
+        <v>401200</v>
       </c>
       <c r="C157" s="366" t="s">
         <v>68</v>
@@ -27010,8 +27010,8 @@
       <c r="A158" s="242" t="s">
         <v>69</v>
       </c>
-      <c r="B158" s="242" t="s">
-        <v>69</v>
+      <c r="B158" s="242">
+        <v>401201</v>
       </c>
       <c r="C158" s="366" t="s">
         <v>70</v>
@@ -27042,8 +27042,8 @@
       <c r="A159" s="243" t="s">
         <v>69</v>
       </c>
-      <c r="B159" s="243" t="s">
-        <v>69</v>
+      <c r="B159" s="243">
+        <v>401201</v>
       </c>
       <c r="C159" s="366" t="s">
         <v>72</v>
@@ -27074,8 +27074,8 @@
       <c r="A160" s="241" t="s">
         <v>74</v>
       </c>
-      <c r="B160" s="241" t="s">
-        <v>74</v>
+      <c r="B160" s="241">
+        <v>401500</v>
       </c>
       <c r="C160" s="171" t="s">
         <v>75</v>
@@ -27106,8 +27106,8 @@
       <c r="A161" s="241" t="s">
         <v>76</v>
       </c>
-      <c r="B161" s="241" t="s">
-        <v>76</v>
+      <c r="B161" s="241">
+        <v>401501</v>
       </c>
       <c r="C161" s="171" t="s">
         <v>77</v>
@@ -27138,8 +27138,8 @@
       <c r="A162" s="241" t="s">
         <v>55</v>
       </c>
-      <c r="B162" s="241" t="s">
-        <v>55</v>
+      <c r="B162" s="241">
+        <v>401590</v>
       </c>
       <c r="C162" s="171" t="s">
         <v>79</v>
@@ -27170,8 +27170,8 @@
       <c r="A163" s="241" t="s">
         <v>80</v>
       </c>
-      <c r="B163" s="241" t="s">
-        <v>80</v>
+      <c r="B163" s="241">
+        <v>401600</v>
       </c>
       <c r="C163" s="171" t="s">
         <v>81</v>
@@ -27202,8 +27202,8 @@
       <c r="A164" s="241" t="s">
         <v>82</v>
       </c>
-      <c r="B164" s="241" t="s">
-        <v>82</v>
+      <c r="B164" s="241">
+        <v>401601</v>
       </c>
       <c r="C164" s="171" t="s">
         <v>83</v>
@@ -27234,8 +27234,8 @@
       <c r="A165" s="242" t="s">
         <v>71</v>
       </c>
-      <c r="B165" s="242" t="s">
-        <v>71</v>
+      <c r="B165" s="242">
+        <v>401700</v>
       </c>
       <c r="C165" s="366" t="s">
         <v>84</v>
@@ -27266,8 +27266,8 @@
       <c r="A166" s="217" t="s">
         <v>85</v>
       </c>
-      <c r="B166" s="217" t="s">
-        <v>85</v>
+      <c r="B166" s="217">
+        <v>401701</v>
       </c>
       <c r="C166" s="182" t="s">
         <v>86</v>
@@ -27298,8 +27298,8 @@
       <c r="A167" s="242" t="s">
         <v>73</v>
       </c>
-      <c r="B167" s="242" t="s">
-        <v>73</v>
+      <c r="B167" s="242">
+        <v>401703</v>
       </c>
       <c r="C167" s="366" t="s">
         <v>87</v>
@@ -27330,8 +27330,8 @@
       <c r="A168" s="241" t="s">
         <v>88</v>
       </c>
-      <c r="B168" s="241" t="s">
-        <v>88</v>
+      <c r="B168" s="241">
+        <v>402100</v>
       </c>
       <c r="C168" s="171" t="s">
         <v>89</v>
@@ -27362,8 +27362,8 @@
       <c r="A169" s="215" t="s">
         <v>78</v>
       </c>
-      <c r="B169" s="215" t="s">
-        <v>78</v>
+      <c r="B169" s="215">
+        <v>402190</v>
       </c>
       <c r="C169" s="171" t="s">
         <v>90</v>
@@ -27394,8 +27394,8 @@
       <c r="A170" s="241" t="s">
         <v>91</v>
       </c>
-      <c r="B170" s="241" t="s">
-        <v>91</v>
+      <c r="B170" s="241">
+        <v>402300</v>
       </c>
       <c r="C170" s="171" t="s">
         <v>92</v>
@@ -27414,8 +27414,8 @@
       <c r="A171" s="241" t="s">
         <v>93</v>
       </c>
-      <c r="B171" s="241" t="s">
-        <v>93</v>
+      <c r="B171" s="241">
+        <v>402390</v>
       </c>
       <c r="C171" s="171" t="s">
         <v>94</v>
@@ -27434,8 +27434,8 @@
       <c r="A172" s="215" t="s">
         <v>95</v>
       </c>
-      <c r="B172" s="215" t="s">
-        <v>95</v>
+      <c r="B172" s="215">
+        <v>402500</v>
       </c>
       <c r="C172" s="171" t="s">
         <v>96</v>
@@ -27454,8 +27454,8 @@
       <c r="A173" s="215" t="s">
         <v>97</v>
       </c>
-      <c r="B173" s="215" t="s">
-        <v>97</v>
+      <c r="B173" s="215">
+        <v>402501</v>
       </c>
       <c r="C173" s="171" t="s">
         <v>98</v>
@@ -27474,8 +27474,8 @@
       <c r="A174" s="241" t="s">
         <v>99</v>
       </c>
-      <c r="B174" s="241" t="s">
-        <v>99</v>
+      <c r="B174" s="241">
+        <v>402700</v>
       </c>
       <c r="C174" s="171" t="s">
         <v>100</v>
@@ -27494,8 +27494,8 @@
       <c r="A175" s="241" t="s">
         <v>101</v>
       </c>
-      <c r="B175" s="241" t="s">
-        <v>101</v>
+      <c r="B175" s="241">
+        <v>402701</v>
       </c>
       <c r="C175" s="171" t="s">
         <v>102</v>
@@ -27514,8 +27514,8 @@
       <c r="A176" s="241" t="s">
         <v>103</v>
       </c>
-      <c r="B176" s="241" t="s">
-        <v>103</v>
+      <c r="B176" s="241">
+        <v>402900</v>
       </c>
       <c r="C176" s="171" t="s">
         <v>104</v>
@@ -27534,8 +27534,8 @@
       <c r="A177" s="241" t="s">
         <v>106</v>
       </c>
-      <c r="B177" s="241" t="s">
-        <v>106</v>
+      <c r="B177" s="241">
+        <v>402901</v>
       </c>
       <c r="C177" s="171" t="s">
         <v>107</v>
@@ -27554,8 +27554,8 @@
       <c r="A178" s="215" t="s">
         <v>108</v>
       </c>
-      <c r="B178" s="215" t="s">
-        <v>108</v>
+      <c r="B178" s="215">
+        <v>403600</v>
       </c>
       <c r="C178" s="171" t="s">
         <v>36</v>
@@ -27574,8 +27574,8 @@
       <c r="A179" s="244" t="s">
         <v>33</v>
       </c>
-      <c r="B179" s="244" t="s">
-        <v>33</v>
+      <c r="B179" s="244">
+        <v>403690</v>
       </c>
       <c r="C179" s="171"/>
       <c r="D179" s="177" t="s">
@@ -27592,8 +27592,8 @@
       <c r="A180" s="215" t="s">
         <v>110</v>
       </c>
-      <c r="B180" s="215" t="s">
-        <v>110</v>
+      <c r="B180" s="215">
+        <v>405600</v>
       </c>
       <c r="C180" s="171" t="s">
         <v>111</v>
@@ -27612,8 +27612,8 @@
       <c r="A181" s="218" t="s">
         <v>112</v>
       </c>
-      <c r="B181" s="218" t="s">
-        <v>112</v>
+      <c r="B181" s="218">
+        <v>405601</v>
       </c>
       <c r="C181" s="367" t="s">
         <v>113</v>
@@ -27632,8 +27632,8 @@
       <c r="A182" s="241" t="s">
         <v>114</v>
       </c>
-      <c r="B182" s="241" t="s">
-        <v>114</v>
+      <c r="B182" s="241">
+        <v>405700</v>
       </c>
       <c r="C182" s="171" t="s">
         <v>115</v>
@@ -27652,8 +27652,8 @@
       <c r="A183" s="241" t="s">
         <v>117</v>
       </c>
-      <c r="B183" s="241" t="s">
-        <v>117</v>
+      <c r="B183" s="241">
+        <v>405701</v>
       </c>
       <c r="C183" s="171" t="s">
         <v>118</v>
@@ -27672,8 +27672,8 @@
       <c r="A184" s="241" t="s">
         <v>119</v>
       </c>
-      <c r="B184" s="241" t="s">
-        <v>119</v>
+      <c r="B184" s="241">
+        <v>405900</v>
       </c>
       <c r="C184" s="171" t="s">
         <v>120</v>
@@ -27692,8 +27692,8 @@
       <c r="A185" s="241" t="s">
         <v>119</v>
       </c>
-      <c r="B185" s="241" t="s">
-        <v>119</v>
+      <c r="B185" s="241">
+        <v>405900</v>
       </c>
       <c r="C185" s="171" t="s">
         <v>121</v>
@@ -27712,8 +27712,8 @@
       <c r="A186" s="241" t="s">
         <v>122</v>
       </c>
-      <c r="B186" s="241" t="s">
-        <v>122</v>
+      <c r="B186" s="241">
+        <v>405901</v>
       </c>
       <c r="C186" s="171" t="s">
         <v>123</v>
@@ -27732,8 +27732,8 @@
       <c r="A187" s="241" t="s">
         <v>122</v>
       </c>
-      <c r="B187" s="241" t="s">
-        <v>122</v>
+      <c r="B187" s="241">
+        <v>405901</v>
       </c>
       <c r="C187" s="171" t="s">
         <v>124</v>
@@ -27752,8 +27752,8 @@
       <c r="A188" s="215" t="s">
         <v>125</v>
       </c>
-      <c r="B188" s="215" t="s">
-        <v>125</v>
+      <c r="B188" s="215">
+        <v>406000</v>
       </c>
       <c r="C188" s="171" t="s">
         <v>40</v>
@@ -27772,8 +27772,8 @@
       <c r="A189" s="218" t="s">
         <v>126</v>
       </c>
-      <c r="B189" s="218" t="s">
-        <v>126</v>
+      <c r="B189" s="218">
+        <v>406006</v>
       </c>
       <c r="C189" s="367" t="s">
         <v>127</v>
@@ -27792,8 +27792,8 @@
       <c r="A190" s="218" t="s">
         <v>128</v>
       </c>
-      <c r="B190" s="218" t="s">
-        <v>128</v>
+      <c r="B190" s="218">
+        <v>406030</v>
       </c>
       <c r="C190" s="367" t="s">
         <v>129</v>
@@ -27812,8 +27812,8 @@
       <c r="A191" s="215" t="s">
         <v>130</v>
       </c>
-      <c r="B191" s="215" t="s">
-        <v>130</v>
+      <c r="B191" s="215">
+        <v>406100</v>
       </c>
       <c r="C191" s="171" t="s">
         <v>131</v>
@@ -27832,8 +27832,8 @@
       <c r="A192" s="215" t="s">
         <v>132</v>
       </c>
-      <c r="B192" s="215" t="s">
-        <v>132</v>
+      <c r="B192" s="215">
+        <v>406106</v>
       </c>
       <c r="C192" s="171" t="s">
         <v>127</v>
@@ -27852,8 +27852,8 @@
       <c r="A193" s="215" t="s">
         <v>132</v>
       </c>
-      <c r="B193" s="215" t="s">
-        <v>132</v>
+      <c r="B193" s="215">
+        <v>406106</v>
       </c>
       <c r="C193" s="171" t="s">
         <v>133</v>
@@ -27872,8 +27872,8 @@
       <c r="A194" s="215" t="s">
         <v>134</v>
       </c>
-      <c r="B194" s="215" t="s">
-        <v>134</v>
+      <c r="B194" s="215">
+        <v>406138</v>
       </c>
       <c r="C194" s="171" t="s">
         <v>129</v>
@@ -27892,8 +27892,8 @@
       <c r="A195" s="215" t="s">
         <v>134</v>
       </c>
-      <c r="B195" s="215" t="s">
-        <v>134</v>
+      <c r="B195" s="215">
+        <v>406138</v>
       </c>
       <c r="C195" s="171" t="s">
         <v>135</v>
@@ -27912,8 +27912,8 @@
       <c r="A196" s="241" t="s">
         <v>63</v>
       </c>
-      <c r="B196" s="241" t="s">
-        <v>63</v>
+      <c r="B196" s="241">
+        <v>406200</v>
       </c>
       <c r="C196" s="171" t="s">
         <v>40</v>
@@ -27932,8 +27932,8 @@
       <c r="A197" s="215" t="s">
         <v>136</v>
       </c>
-      <c r="B197" s="215" t="s">
-        <v>136</v>
+      <c r="B197" s="215">
+        <v>406206</v>
       </c>
       <c r="C197" s="171" t="s">
         <v>137</v>
@@ -27952,8 +27952,8 @@
       <c r="A198" s="241" t="s">
         <v>66</v>
       </c>
-      <c r="B198" s="241" t="s">
-        <v>66</v>
+      <c r="B198" s="241">
+        <v>406209</v>
       </c>
       <c r="C198" s="171"/>
       <c r="D198" s="177" t="s">
@@ -27970,8 +27970,8 @@
       <c r="A199" s="215" t="s">
         <v>139</v>
       </c>
-      <c r="B199" s="215" t="s">
-        <v>139</v>
+      <c r="B199" s="215">
+        <v>406238</v>
       </c>
       <c r="C199" s="171" t="s">
         <v>140</v>
@@ -27990,8 +27990,8 @@
       <c r="A200" s="241" t="s">
         <v>35</v>
       </c>
-      <c r="B200" s="241" t="s">
-        <v>35</v>
+      <c r="B200" s="241">
+        <v>406300</v>
       </c>
       <c r="C200" s="171" t="s">
         <v>142</v>
@@ -28010,8 +28010,8 @@
       <c r="A201" s="245" t="s">
         <v>143</v>
       </c>
-      <c r="B201" s="245" t="s">
-        <v>143</v>
+      <c r="B201" s="245">
+        <v>406301</v>
       </c>
       <c r="C201" s="171" t="s">
         <v>144</v>
@@ -28030,8 +28030,8 @@
       <c r="A202" s="245" t="s">
         <v>145</v>
       </c>
-      <c r="B202" s="245" t="s">
-        <v>145</v>
+      <c r="B202" s="245">
+        <v>406401</v>
       </c>
       <c r="C202" s="171" t="s">
         <v>146</v>
@@ -28050,8 +28050,8 @@
       <c r="A203" s="219" t="s">
         <v>147</v>
       </c>
-      <c r="B203" s="219" t="s">
-        <v>147</v>
+      <c r="B203" s="219">
+        <v>406500</v>
       </c>
       <c r="C203" s="171" t="s">
         <v>148</v>
@@ -28070,8 +28070,8 @@
       <c r="A204" s="219" t="s">
         <v>149</v>
       </c>
-      <c r="B204" s="219" t="s">
-        <v>149</v>
+      <c r="B204" s="219">
+        <v>406506</v>
       </c>
       <c r="C204" s="171" t="s">
         <v>150</v>
@@ -28090,8 +28090,8 @@
       <c r="A205" s="219" t="s">
         <v>151</v>
       </c>
-      <c r="B205" s="219" t="s">
-        <v>151</v>
+      <c r="B205" s="219">
+        <v>406538</v>
       </c>
       <c r="C205" s="171" t="s">
         <v>152</v>
@@ -28110,8 +28110,8 @@
       <c r="A206" s="219" t="s">
         <v>153</v>
       </c>
-      <c r="B206" s="219" t="s">
-        <v>153</v>
+      <c r="B206" s="219">
+        <v>406560</v>
       </c>
       <c r="C206" s="171" t="s">
         <v>154</v>
@@ -28130,8 +28130,8 @@
       <c r="A207" s="219" t="s">
         <v>155</v>
       </c>
-      <c r="B207" s="219" t="s">
-        <v>155</v>
+      <c r="B207" s="219">
+        <v>406630</v>
       </c>
       <c r="C207" s="171"/>
       <c r="D207" s="170"/>
@@ -28142,8 +28142,8 @@
       <c r="A208" s="219" t="s">
         <v>156</v>
       </c>
-      <c r="B208" s="219" t="s">
-        <v>156</v>
+      <c r="B208" s="219">
+        <v>406660</v>
       </c>
       <c r="C208" s="171" t="s">
         <v>157</v>
@@ -28162,8 +28162,8 @@
       <c r="A209" s="219" t="s">
         <v>158</v>
       </c>
-      <c r="B209" s="219" t="s">
-        <v>158</v>
+      <c r="B209" s="219">
+        <v>406760</v>
       </c>
       <c r="C209" s="171" t="s">
         <v>159</v>
@@ -28182,8 +28182,8 @@
       <c r="A210" s="220" t="s">
         <v>160</v>
       </c>
-      <c r="B210" s="220" t="s">
-        <v>160</v>
+      <c r="B210" s="220">
+        <v>407038</v>
       </c>
       <c r="C210" s="182" t="s">
         <v>161</v>
@@ -28218,8 +28218,8 @@
       <c r="A212" s="219" t="s">
         <v>162</v>
       </c>
-      <c r="B212" s="219" t="s">
-        <v>162</v>
+      <c r="B212" s="219">
+        <v>407100</v>
       </c>
       <c r="C212" s="171" t="s">
         <v>163</v>
@@ -28236,8 +28236,8 @@
       <c r="A213" s="219" t="s">
         <v>166</v>
       </c>
-      <c r="B213" s="219" t="s">
-        <v>166</v>
+      <c r="B213" s="219">
+        <v>407101</v>
       </c>
       <c r="C213" s="171" t="s">
         <v>167</v>
@@ -28254,8 +28254,8 @@
       <c r="A214" s="219" t="s">
         <v>168</v>
       </c>
-      <c r="B214" s="219" t="s">
-        <v>168</v>
+      <c r="B214" s="219">
+        <v>407301</v>
       </c>
       <c r="C214" s="171" t="s">
         <v>169</v>
@@ -28268,8 +28268,8 @@
       <c r="A215" s="219" t="s">
         <v>170</v>
       </c>
-      <c r="B215" s="219" t="s">
-        <v>170</v>
+      <c r="B215" s="219">
+        <v>407300</v>
       </c>
       <c r="C215" s="171" t="s">
         <v>171</v>
@@ -28282,8 +28282,8 @@
       <c r="A216" s="219" t="s">
         <v>172</v>
       </c>
-      <c r="B216" s="219" t="s">
-        <v>172</v>
+      <c r="B216" s="219">
+        <v>407201</v>
       </c>
       <c r="C216" s="171" t="s">
         <v>173</v>
@@ -28296,8 +28296,8 @@
       <c r="A217" s="219" t="s">
         <v>174</v>
       </c>
-      <c r="B217" s="219" t="s">
-        <v>174</v>
+      <c r="B217" s="219">
+        <v>407200</v>
       </c>
       <c r="C217" s="171" t="s">
         <v>175</v>
@@ -28311,7 +28311,7 @@
         <v>4074</v>
       </c>
       <c r="B218" s="219">
-        <v>4074</v>
+        <v>407400</v>
       </c>
       <c r="C218" s="171" t="s">
         <v>176</v>
@@ -28327,7 +28327,7 @@
         <v>4101</v>
       </c>
       <c r="B219" s="206">
-        <v>4101</v>
+        <v>410100</v>
       </c>
       <c r="C219" s="62" t="s">
         <v>178</v>
@@ -28346,8 +28346,8 @@
       <c r="A220" s="219" t="s">
         <v>181</v>
       </c>
-      <c r="B220" s="219" t="s">
-        <v>181</v>
+      <c r="B220" s="219">
+        <v>383460</v>
       </c>
       <c r="C220" s="171" t="s">
         <v>182</v>
@@ -28366,8 +28366,8 @@
       <c r="A221" s="220" t="s">
         <v>184</v>
       </c>
-      <c r="B221" s="220" t="s">
-        <v>184</v>
+      <c r="B221" s="220">
+        <v>412401</v>
       </c>
       <c r="C221" s="368" t="s">
         <v>185</v>
@@ -28386,8 +28386,8 @@
       <c r="A222" s="219" t="s">
         <v>187</v>
       </c>
-      <c r="B222" s="219" t="s">
-        <v>187</v>
+      <c r="B222" s="219">
+        <v>412500</v>
       </c>
       <c r="C222" s="171" t="s">
         <v>188</v>
@@ -28406,8 +28406,8 @@
       <c r="A223" s="220" t="s">
         <v>189</v>
       </c>
-      <c r="B223" s="220" t="s">
-        <v>189</v>
+      <c r="B223" s="220">
+        <v>413501</v>
       </c>
       <c r="C223" s="368" t="s">
         <v>190</v>
@@ -28426,8 +28426,8 @@
       <c r="A224" s="220" t="s">
         <v>193</v>
       </c>
-      <c r="B224" s="220" t="s">
-        <v>193</v>
+      <c r="B224" s="220">
+        <v>413560</v>
       </c>
       <c r="C224" s="368" t="s">
         <v>194</v>
@@ -28446,8 +28446,8 @@
       <c r="A225" s="220" t="s">
         <v>195</v>
       </c>
-      <c r="B225" s="220" t="s">
-        <v>195</v>
+      <c r="B225" s="220">
+        <v>413561</v>
       </c>
       <c r="C225" s="368" t="s">
         <v>196</v>
@@ -28466,8 +28466,8 @@
       <c r="A226" s="220" t="s">
         <v>197</v>
       </c>
-      <c r="B226" s="220" t="s">
-        <v>197</v>
+      <c r="B226" s="220">
+        <v>414261</v>
       </c>
       <c r="C226" s="368" t="s">
         <v>198</v>
@@ -28486,8 +28486,8 @@
       <c r="A227" s="220" t="s">
         <v>200</v>
       </c>
-      <c r="B227" s="220" t="s">
-        <v>200</v>
+      <c r="B227" s="220">
+        <v>414760</v>
       </c>
       <c r="C227" s="369" t="s">
         <v>201</v>
@@ -28506,8 +28506,8 @@
       <c r="A228" s="220" t="s">
         <v>202</v>
       </c>
-      <c r="B228" s="220" t="s">
-        <v>202</v>
+      <c r="B228" s="220">
+        <v>414800</v>
       </c>
       <c r="C228" s="369" t="s">
         <v>203</v>
@@ -28526,8 +28526,8 @@
       <c r="A229" s="220" t="s">
         <v>204</v>
       </c>
-      <c r="B229" s="220" t="s">
-        <v>204</v>
+      <c r="B229" s="220">
+        <v>414806</v>
       </c>
       <c r="C229" s="368" t="s">
         <v>205</v>
@@ -28546,8 +28546,8 @@
       <c r="A230" s="220" t="s">
         <v>206</v>
       </c>
-      <c r="B230" s="220" t="s">
-        <v>206</v>
+      <c r="B230" s="220">
+        <v>414838</v>
       </c>
       <c r="C230" s="369" t="s">
         <v>207</v>
@@ -28566,8 +28566,8 @@
       <c r="A231" s="220" t="s">
         <v>208</v>
       </c>
-      <c r="B231" s="220" t="s">
-        <v>208</v>
+      <c r="B231" s="220">
+        <v>414860</v>
       </c>
       <c r="C231" s="368" t="s">
         <v>209</v>
@@ -28586,8 +28586,8 @@
       <c r="A232" s="220" t="s">
         <v>208</v>
       </c>
-      <c r="B232" s="220" t="s">
-        <v>208</v>
+      <c r="B232" s="220">
+        <v>414860</v>
       </c>
       <c r="C232" s="369" t="s">
         <v>203</v>
@@ -28606,8 +28606,8 @@
       <c r="A233" s="220" t="s">
         <v>210</v>
       </c>
-      <c r="B233" s="220" t="s">
-        <v>210</v>
+      <c r="B233" s="220">
+        <v>414960</v>
       </c>
       <c r="C233" s="368" t="s">
         <v>211</v>
@@ -28626,8 +28626,8 @@
       <c r="A234" s="220" t="s">
         <v>212</v>
       </c>
-      <c r="B234" s="220" t="s">
-        <v>212</v>
+      <c r="B234" s="220">
+        <v>415700</v>
       </c>
       <c r="C234" s="368" t="s">
         <v>213</v>
@@ -28646,8 +28646,8 @@
       <c r="A235" s="220" t="s">
         <v>214</v>
       </c>
-      <c r="B235" s="220" t="s">
-        <v>214</v>
+      <c r="B235" s="220">
+        <v>415701</v>
       </c>
       <c r="C235" s="368" t="s">
         <v>215</v>
@@ -28666,8 +28666,8 @@
       <c r="A236" s="220" t="s">
         <v>216</v>
       </c>
-      <c r="B236" s="220" t="s">
-        <v>216</v>
+      <c r="B236" s="220">
+        <v>416900</v>
       </c>
       <c r="C236" s="369" t="s">
         <v>217</v>
@@ -28686,8 +28686,8 @@
       <c r="A237" s="220" t="s">
         <v>218</v>
       </c>
-      <c r="B237" s="220" t="s">
-        <v>218</v>
+      <c r="B237" s="220">
+        <v>416901</v>
       </c>
       <c r="C237" s="368" t="s">
         <v>219</v>
@@ -28706,8 +28706,8 @@
       <c r="A238" s="220" t="s">
         <v>218</v>
       </c>
-      <c r="B238" s="220" t="s">
-        <v>218</v>
+      <c r="B238" s="220">
+        <v>416901</v>
       </c>
       <c r="C238" s="369" t="s">
         <v>220</v>
@@ -28726,8 +28726,8 @@
       <c r="A239" s="220" t="s">
         <v>221</v>
       </c>
-      <c r="B239" s="220" t="s">
-        <v>221</v>
+      <c r="B239" s="220">
+        <v>417000</v>
       </c>
       <c r="C239" s="369" t="s">
         <v>222</v>
@@ -28746,8 +28746,8 @@
       <c r="A240" s="220" t="s">
         <v>223</v>
       </c>
-      <c r="B240" s="220" t="s">
-        <v>223</v>
+      <c r="B240" s="220">
+        <v>417001</v>
       </c>
       <c r="C240" s="368" t="s">
         <v>224</v>
@@ -28766,8 +28766,8 @@
       <c r="A241" s="220" t="s">
         <v>225</v>
       </c>
-      <c r="B241" s="220" t="s">
-        <v>225</v>
+      <c r="B241" s="220">
+        <v>417100</v>
       </c>
       <c r="C241" s="368" t="s">
         <v>226</v>
@@ -28786,8 +28786,8 @@
       <c r="A242" s="220" t="s">
         <v>227</v>
       </c>
-      <c r="B242" s="220" t="s">
-        <v>227</v>
+      <c r="B242" s="220">
+        <v>418060</v>
       </c>
       <c r="C242" s="368" t="s">
         <v>228</v>
@@ -28807,7 +28807,7 @@
         <v>4106</v>
       </c>
       <c r="B243" s="206">
-        <v>4106</v>
+        <v>410600</v>
       </c>
       <c r="C243" s="370" t="s">
         <v>229</v>
@@ -28827,7 +28827,7 @@
         <v>4108</v>
       </c>
       <c r="B244" s="206">
-        <v>4108</v>
+        <v>410800</v>
       </c>
       <c r="C244" s="62" t="s">
         <v>230</v>
@@ -28847,7 +28847,7 @@
         <v>4108</v>
       </c>
       <c r="B245" s="206">
-        <v>4108</v>
+        <v>410800</v>
       </c>
       <c r="C245" s="370" t="s">
         <v>231</v>
@@ -28867,7 +28867,7 @@
         <v>4109</v>
       </c>
       <c r="B246" s="206">
-        <v>4109</v>
+        <v>410900</v>
       </c>
       <c r="C246" s="62" t="s">
         <v>233</v>
@@ -28887,7 +28887,7 @@
         <v>4109</v>
       </c>
       <c r="B247" s="206">
-        <v>4109</v>
+        <v>410900</v>
       </c>
       <c r="C247" s="370" t="s">
         <v>234</v>
@@ -28907,7 +28907,7 @@
         <v>4110</v>
       </c>
       <c r="B248" s="206">
-        <v>4110</v>
+        <v>411000</v>
       </c>
       <c r="C248" s="370" t="s">
         <v>236</v>
@@ -28927,7 +28927,7 @@
         <v>4113</v>
       </c>
       <c r="B249" s="206">
-        <v>4113</v>
+        <v>411300</v>
       </c>
       <c r="C249" s="62" t="s">
         <v>237</v>
@@ -28947,7 +28947,7 @@
         <v>4113</v>
       </c>
       <c r="B250" s="206">
-        <v>4113</v>
+        <v>411300</v>
       </c>
       <c r="C250" s="370" t="s">
         <v>238</v>
@@ -28967,7 +28967,7 @@
         <v>4116</v>
       </c>
       <c r="B251" s="206">
-        <v>4116</v>
+        <v>411600</v>
       </c>
       <c r="C251" s="62" t="s">
         <v>240</v>
@@ -28987,7 +28987,7 @@
         <v>4119</v>
       </c>
       <c r="B252" s="206">
-        <v>4119</v>
+        <v>411900</v>
       </c>
       <c r="C252" s="62" t="s">
         <v>243</v>
@@ -29007,7 +29007,7 @@
         <v>4120</v>
       </c>
       <c r="B253" s="206">
-        <v>4120</v>
+        <v>412000</v>
       </c>
       <c r="C253" s="62" t="s">
         <v>244</v>
@@ -29027,7 +29027,7 @@
         <v>4121</v>
       </c>
       <c r="B254" s="206">
-        <v>4121</v>
+        <v>412100</v>
       </c>
       <c r="C254" s="62" t="s">
         <v>247</v>
@@ -29047,7 +29047,7 @@
         <v>4122</v>
       </c>
       <c r="B255" s="206">
-        <v>4122</v>
+        <v>412200</v>
       </c>
       <c r="C255" s="62" t="s">
         <v>248</v>
@@ -29067,7 +29067,7 @@
         <v>4123</v>
       </c>
       <c r="B256" s="206">
-        <v>4123</v>
+        <v>412300</v>
       </c>
       <c r="C256" s="62" t="s">
         <v>249</v>
@@ -29086,8 +29086,8 @@
       <c r="A257" s="206" t="s">
         <v>250</v>
       </c>
-      <c r="B257" s="206" t="s">
-        <v>250</v>
+      <c r="B257" s="206">
+        <v>412400</v>
       </c>
       <c r="C257" s="370" t="s">
         <v>251</v>
@@ -29107,7 +29107,7 @@
         <v>4128</v>
       </c>
       <c r="B258" s="206">
-        <v>4128</v>
+        <v>412800</v>
       </c>
       <c r="C258" s="62" t="s">
         <v>252</v>
@@ -29127,7 +29127,7 @@
         <v>4130</v>
       </c>
       <c r="B259" s="206">
-        <v>4130</v>
+        <v>413000</v>
       </c>
       <c r="C259" s="62" t="s">
         <v>253</v>
@@ -29147,7 +29147,7 @@
         <v>4135</v>
       </c>
       <c r="B260" s="206">
-        <v>4135</v>
+        <v>413500</v>
       </c>
       <c r="C260" s="370" t="s">
         <v>254</v>
@@ -29167,7 +29167,7 @@
         <v>4136</v>
       </c>
       <c r="B261" s="206">
-        <v>4136</v>
+        <v>413600</v>
       </c>
       <c r="C261" s="62" t="s">
         <v>255</v>
@@ -29187,7 +29187,7 @@
         <v>4137</v>
       </c>
       <c r="B262" s="206">
-        <v>4137</v>
+        <v>413700</v>
       </c>
       <c r="C262" s="62" t="s">
         <v>257</v>
@@ -29207,7 +29207,7 @@
         <v>4149</v>
       </c>
       <c r="B263" s="206">
-        <v>4149</v>
+        <v>414900</v>
       </c>
       <c r="C263" s="370" t="s">
         <v>258</v>
@@ -29227,7 +29227,7 @@
         <v>4153</v>
       </c>
       <c r="B264" s="206">
-        <v>4153</v>
+        <v>415300</v>
       </c>
       <c r="C264" s="62" t="s">
         <v>261</v>
@@ -29246,8 +29246,8 @@
       <c r="A265" s="206" t="s">
         <v>262</v>
       </c>
-      <c r="B265" s="206" t="s">
-        <v>262</v>
+      <c r="B265" s="206">
+        <v>415500</v>
       </c>
       <c r="C265" s="370" t="s">
         <v>263</v>
@@ -29266,8 +29266,8 @@
       <c r="A266" s="206" t="s">
         <v>265</v>
       </c>
-      <c r="B266" s="206" t="s">
-        <v>265</v>
+      <c r="B266" s="206">
+        <v>415501</v>
       </c>
       <c r="C266" s="370" t="s">
         <v>266</v>
@@ -29287,7 +29287,7 @@
         <v>4158</v>
       </c>
       <c r="B267" s="206">
-        <v>4158</v>
+        <v>415800</v>
       </c>
       <c r="C267" s="62" t="s">
         <v>267</v>
@@ -29307,7 +29307,7 @@
         <v>4160</v>
       </c>
       <c r="B268" s="206">
-        <v>4160</v>
+        <v>416000</v>
       </c>
       <c r="C268" s="370" t="s">
         <v>268</v>
@@ -29327,7 +29327,7 @@
         <v>4165</v>
       </c>
       <c r="B269" s="206">
-        <v>4165</v>
+        <v>416500</v>
       </c>
       <c r="C269" s="62" t="s">
         <v>269</v>
@@ -29347,7 +29347,7 @@
         <v>4166</v>
       </c>
       <c r="B270" s="206">
-        <v>4166</v>
+        <v>416600</v>
       </c>
       <c r="C270" s="62" t="s">
         <v>270</v>
@@ -29367,7 +29367,7 @@
         <v>4166</v>
       </c>
       <c r="B271" s="206">
-        <v>4166</v>
+        <v>416600</v>
       </c>
       <c r="C271" s="370" t="s">
         <v>271</v>
@@ -29395,7 +29395,7 @@
         <v>4168</v>
       </c>
       <c r="B272" s="204">
-        <v>4168</v>
+        <v>416800</v>
       </c>
       <c r="C272" s="371" t="s">
         <v>272</v>
@@ -29423,7 +29423,7 @@
         <v>4168</v>
       </c>
       <c r="B273" s="204">
-        <v>4168</v>
+        <v>416800</v>
       </c>
       <c r="C273" s="372"/>
       <c r="D273" s="200"/>
@@ -29447,7 +29447,7 @@
         <v>4176</v>
       </c>
       <c r="B274" s="204">
-        <v>4176</v>
+        <v>417600</v>
       </c>
       <c r="C274" s="371" t="s">
         <v>252</v>
@@ -29475,7 +29475,7 @@
         <v>4176</v>
       </c>
       <c r="B275" s="204">
-        <v>4176</v>
+        <v>417600</v>
       </c>
       <c r="C275" s="372" t="s">
         <v>273</v>
@@ -29503,7 +29503,7 @@
         <v>4177</v>
       </c>
       <c r="B276" s="204">
-        <v>4177</v>
+        <v>417700</v>
       </c>
       <c r="C276" s="372" t="s">
         <v>201</v>
@@ -29531,7 +29531,7 @@
         <v>4178</v>
       </c>
       <c r="B277" s="204">
-        <v>4178</v>
+        <v>417800</v>
       </c>
       <c r="C277" s="372" t="s">
         <v>274</v>
@@ -29559,7 +29559,7 @@
         <v>4179</v>
       </c>
       <c r="B278" s="204">
-        <v>4179</v>
+        <v>417900</v>
       </c>
       <c r="C278" s="372" t="s">
         <v>275</v>
@@ -29585,7 +29585,7 @@
         <v>4183</v>
       </c>
       <c r="B279" s="204">
-        <v>4183</v>
+        <v>418300</v>
       </c>
       <c r="C279" s="371" t="s">
         <v>276</v>
@@ -29613,7 +29613,7 @@
         <v>4185</v>
       </c>
       <c r="B280" s="251">
-        <v>4185</v>
+        <v>418500</v>
       </c>
       <c r="C280" s="373" t="s">
         <v>278</v>
@@ -29658,8 +29658,8 @@
       <c r="A282" s="260" t="s">
         <v>280</v>
       </c>
-      <c r="B282" s="260" t="s">
-        <v>280</v>
+      <c r="B282" s="260">
+        <v>420101</v>
       </c>
       <c r="C282" s="258" t="s">
         <v>281</v>
@@ -29686,8 +29686,8 @@
       <c r="A283" s="261" t="s">
         <v>282</v>
       </c>
-      <c r="B283" s="261" t="s">
-        <v>282</v>
+      <c r="B283" s="261">
+        <v>420160</v>
       </c>
       <c r="C283" s="258" t="s">
         <v>283</v>
@@ -29714,8 +29714,8 @@
       <c r="A284" s="261" t="s">
         <v>284</v>
       </c>
-      <c r="B284" s="261" t="s">
-        <v>284</v>
+      <c r="B284" s="261">
+        <v>420100</v>
       </c>
       <c r="C284" s="258" t="s">
         <v>285</v>
@@ -29742,8 +29742,8 @@
       <c r="A285" s="261" t="s">
         <v>286</v>
       </c>
-      <c r="B285" s="261" t="s">
-        <v>286</v>
+      <c r="B285" s="261">
+        <v>420200</v>
       </c>
       <c r="C285" s="258" t="s">
         <v>287</v>
@@ -29770,8 +29770,8 @@
       <c r="A286" s="261" t="s">
         <v>288</v>
       </c>
-      <c r="B286" s="261" t="s">
-        <v>288</v>
+      <c r="B286" s="261">
+        <v>420300</v>
       </c>
       <c r="C286" s="258" t="s">
         <v>289</v>
@@ -29798,8 +29798,8 @@
       <c r="A287" s="261" t="s">
         <v>290</v>
       </c>
-      <c r="B287" s="261" t="s">
-        <v>290</v>
+      <c r="B287" s="261">
+        <v>420301</v>
       </c>
       <c r="C287" s="258" t="s">
         <v>291</v>
@@ -29826,8 +29826,8 @@
       <c r="A288" s="261" t="s">
         <v>292</v>
       </c>
-      <c r="B288" s="261" t="s">
-        <v>292</v>
+      <c r="B288" s="261">
+        <v>420400</v>
       </c>
       <c r="C288" s="258" t="s">
         <v>293</v>
@@ -29854,8 +29854,8 @@
       <c r="A289" s="261" t="s">
         <v>295</v>
       </c>
-      <c r="B289" s="261" t="s">
-        <v>295</v>
+      <c r="B289" s="261">
+        <v>420401</v>
       </c>
       <c r="C289" s="258" t="s">
         <v>296</v>
@@ -29882,8 +29882,8 @@
       <c r="A290" s="261" t="s">
         <v>297</v>
       </c>
-      <c r="B290" s="261" t="s">
-        <v>297</v>
+      <c r="B290" s="261">
+        <v>420402</v>
       </c>
       <c r="C290" s="258" t="s">
         <v>298</v>
@@ -29910,8 +29910,8 @@
       <c r="A291" s="261" t="s">
         <v>299</v>
       </c>
-      <c r="B291" s="261" t="s">
-        <v>299</v>
+      <c r="B291" s="261">
+        <v>420500</v>
       </c>
       <c r="C291" s="258" t="s">
         <v>300</v>
@@ -29938,8 +29938,8 @@
       <c r="A292" s="261" t="s">
         <v>301</v>
       </c>
-      <c r="B292" s="261" t="s">
-        <v>301</v>
+      <c r="B292" s="261">
+        <v>420501</v>
       </c>
       <c r="C292" s="258" t="s">
         <v>302</v>
@@ -29966,8 +29966,8 @@
       <c r="A293" s="261" t="s">
         <v>303</v>
       </c>
-      <c r="B293" s="261" t="s">
-        <v>303</v>
+      <c r="B293" s="261">
+        <v>420600</v>
       </c>
       <c r="C293" s="258" t="s">
         <v>304</v>
@@ -29994,8 +29994,8 @@
       <c r="A294" s="261" t="s">
         <v>305</v>
       </c>
-      <c r="B294" s="261" t="s">
-        <v>305</v>
+      <c r="B294" s="261">
+        <v>420800</v>
       </c>
       <c r="C294" s="258" t="s">
         <v>306</v>
@@ -30022,8 +30022,8 @@
       <c r="A295" s="261" t="s">
         <v>307</v>
       </c>
-      <c r="B295" s="261" t="s">
-        <v>307</v>
+      <c r="B295" s="261">
+        <v>420801</v>
       </c>
       <c r="C295" s="258" t="s">
         <v>308</v>
@@ -30050,8 +30050,8 @@
       <c r="A296" s="261" t="s">
         <v>309</v>
       </c>
-      <c r="B296" s="261" t="s">
-        <v>309</v>
+      <c r="B296" s="261">
+        <v>420802</v>
       </c>
       <c r="C296" s="258" t="s">
         <v>310</v>
@@ -30078,8 +30078,8 @@
       <c r="A297" s="261" t="s">
         <v>311</v>
       </c>
-      <c r="B297" s="261" t="s">
-        <v>311</v>
+      <c r="B297" s="261">
+        <v>420900</v>
       </c>
       <c r="C297" s="258" t="s">
         <v>312</v>
@@ -30106,8 +30106,8 @@
       <c r="A298" s="261" t="s">
         <v>313</v>
       </c>
-      <c r="B298" s="261" t="s">
-        <v>313</v>
+      <c r="B298" s="261">
+        <v>421000</v>
       </c>
       <c r="C298" s="258" t="s">
         <v>314</v>
@@ -30134,8 +30134,8 @@
       <c r="A299" s="261" t="s">
         <v>315</v>
       </c>
-      <c r="B299" s="261" t="s">
-        <v>315</v>
+      <c r="B299" s="261">
+        <v>421001</v>
       </c>
       <c r="C299" s="258" t="s">
         <v>316</v>
@@ -30162,8 +30162,8 @@
       <c r="A300" s="261" t="s">
         <v>317</v>
       </c>
-      <c r="B300" s="261" t="s">
-        <v>317</v>
+      <c r="B300" s="261">
+        <v>421100</v>
       </c>
       <c r="C300" s="258" t="s">
         <v>318</v>
@@ -30190,8 +30190,8 @@
       <c r="A301" s="261" t="s">
         <v>319</v>
       </c>
-      <c r="B301" s="261" t="s">
-        <v>319</v>
+      <c r="B301" s="261">
+        <v>421101</v>
       </c>
       <c r="C301" s="258" t="s">
         <v>320</v>
@@ -30218,8 +30218,8 @@
       <c r="A302" s="261" t="s">
         <v>321</v>
       </c>
-      <c r="B302" s="261" t="s">
-        <v>321</v>
+      <c r="B302" s="261">
+        <v>421300</v>
       </c>
       <c r="C302" s="258" t="s">
         <v>322</v>
@@ -30246,8 +30246,8 @@
       <c r="A303" s="261" t="s">
         <v>323</v>
       </c>
-      <c r="B303" s="261" t="s">
-        <v>323</v>
+      <c r="B303" s="261">
+        <v>421301</v>
       </c>
       <c r="C303" s="258" t="s">
         <v>324</v>
@@ -30266,8 +30266,8 @@
       <c r="A304" s="261" t="s">
         <v>325</v>
       </c>
-      <c r="B304" s="261" t="s">
-        <v>325</v>
+      <c r="B304" s="261">
+        <v>421400</v>
       </c>
       <c r="C304" s="258" t="s">
         <v>326</v>
@@ -30286,8 +30286,8 @@
       <c r="A305" s="261" t="s">
         <v>327</v>
       </c>
-      <c r="B305" s="261" t="s">
-        <v>327</v>
+      <c r="B305" s="261">
+        <v>421401</v>
       </c>
       <c r="C305" s="258" t="s">
         <v>328</v>
@@ -30306,8 +30306,8 @@
       <c r="A306" s="261" t="s">
         <v>329</v>
       </c>
-      <c r="B306" s="261" t="s">
-        <v>329</v>
+      <c r="B306" s="261">
+        <v>421460</v>
       </c>
       <c r="C306" s="258" t="s">
         <v>330</v>
@@ -30326,8 +30326,8 @@
       <c r="A307" s="261" t="s">
         <v>331</v>
       </c>
-      <c r="B307" s="261" t="s">
-        <v>331</v>
+      <c r="B307" s="261">
+        <v>421402</v>
       </c>
       <c r="C307" s="258" t="s">
         <v>332</v>
@@ -30346,8 +30346,8 @@
       <c r="A308" s="261" t="s">
         <v>333</v>
       </c>
-      <c r="B308" s="261" t="s">
-        <v>333</v>
+      <c r="B308" s="261">
+        <v>421600</v>
       </c>
       <c r="C308" s="258" t="s">
         <v>334</v>
@@ -30366,8 +30366,8 @@
       <c r="A309" s="261" t="s">
         <v>335</v>
       </c>
-      <c r="B309" s="261" t="s">
-        <v>335</v>
+      <c r="B309" s="261">
+        <v>421700</v>
       </c>
       <c r="C309" s="258" t="s">
         <v>336</v>
@@ -30386,8 +30386,8 @@
       <c r="A310" s="261" t="s">
         <v>337</v>
       </c>
-      <c r="B310" s="261" t="s">
-        <v>337</v>
+      <c r="B310" s="261">
+        <v>421800</v>
       </c>
       <c r="C310" s="258" t="s">
         <v>338</v>
@@ -30406,8 +30406,8 @@
       <c r="A311" s="261" t="s">
         <v>339</v>
       </c>
-      <c r="B311" s="261" t="s">
-        <v>339</v>
+      <c r="B311" s="261">
+        <v>421801</v>
       </c>
       <c r="C311" s="258" t="s">
         <v>340</v>
@@ -30426,8 +30426,8 @@
       <c r="A312" s="261" t="s">
         <v>341</v>
       </c>
-      <c r="B312" s="261" t="s">
-        <v>341</v>
+      <c r="B312" s="261">
+        <v>421900</v>
       </c>
       <c r="C312" s="258" t="s">
         <v>342</v>
@@ -30446,8 +30446,8 @@
       <c r="A313" s="261" t="s">
         <v>343</v>
       </c>
-      <c r="B313" s="261" t="s">
-        <v>343</v>
+      <c r="B313" s="261">
+        <v>421901</v>
       </c>
       <c r="C313" s="258" t="s">
         <v>342</v>
@@ -30466,8 +30466,8 @@
       <c r="A314" s="261" t="s">
         <v>344</v>
       </c>
-      <c r="B314" s="261" t="s">
-        <v>344</v>
+      <c r="B314" s="261">
+        <v>421902</v>
       </c>
       <c r="C314" s="258" t="s">
         <v>345</v>
@@ -30486,8 +30486,8 @@
       <c r="A315" s="261" t="s">
         <v>346</v>
       </c>
-      <c r="B315" s="261" t="s">
-        <v>346</v>
+      <c r="B315" s="261">
+        <v>422000</v>
       </c>
       <c r="C315" s="258" t="s">
         <v>347</v>
@@ -30506,8 +30506,8 @@
       <c r="A316" s="261" t="s">
         <v>348</v>
       </c>
-      <c r="B316" s="261" t="s">
-        <v>348</v>
+      <c r="B316" s="261">
+        <v>422100</v>
       </c>
       <c r="C316" s="258" t="s">
         <v>349</v>
@@ -30526,8 +30526,8 @@
       <c r="A317" s="261" t="s">
         <v>350</v>
       </c>
-      <c r="B317" s="261" t="s">
-        <v>350</v>
+      <c r="B317" s="261">
+        <v>422101</v>
       </c>
       <c r="C317" s="258" t="s">
         <v>351</v>
@@ -30546,8 +30546,8 @@
       <c r="A318" s="261" t="s">
         <v>352</v>
       </c>
-      <c r="B318" s="261" t="s">
-        <v>352</v>
+      <c r="B318" s="261">
+        <v>422190</v>
       </c>
       <c r="C318" s="258" t="s">
         <v>353</v>
@@ -30566,8 +30566,8 @@
       <c r="A319" s="261" t="s">
         <v>354</v>
       </c>
-      <c r="B319" s="261" t="s">
-        <v>354</v>
+      <c r="B319" s="261">
+        <v>422200</v>
       </c>
       <c r="C319" s="258" t="s">
         <v>355</v>
@@ -30587,7 +30587,7 @@
         <v>4223</v>
       </c>
       <c r="B320" s="261">
-        <v>4223</v>
+        <v>422300</v>
       </c>
       <c r="C320" s="258" t="s">
         <v>356</v>
@@ -30606,8 +30606,8 @@
       <c r="A321" s="261" t="s">
         <v>357</v>
       </c>
-      <c r="B321" s="261" t="s">
-        <v>357</v>
+      <c r="B321" s="261">
+        <v>422400</v>
       </c>
       <c r="C321" s="258" t="s">
         <v>358</v>
@@ -30626,8 +30626,8 @@
       <c r="A322" s="261" t="s">
         <v>359</v>
       </c>
-      <c r="B322" s="261" t="s">
-        <v>359</v>
+      <c r="B322" s="261">
+        <v>422401</v>
       </c>
       <c r="C322" s="258" t="s">
         <v>360</v>
@@ -30646,8 +30646,8 @@
       <c r="A323" s="261" t="s">
         <v>361</v>
       </c>
-      <c r="B323" s="261" t="s">
-        <v>361</v>
+      <c r="B323" s="261">
+        <v>422500</v>
       </c>
       <c r="C323" s="258" t="s">
         <v>362</v>
@@ -30666,8 +30666,8 @@
       <c r="A324" s="261" t="s">
         <v>363</v>
       </c>
-      <c r="B324" s="261" t="s">
-        <v>363</v>
+      <c r="B324" s="261">
+        <v>422501</v>
       </c>
       <c r="C324" s="258" t="s">
         <v>364</v>
@@ -30687,7 +30687,7 @@
         <v>4226</v>
       </c>
       <c r="B325" s="261">
-        <v>4226</v>
+        <v>422600</v>
       </c>
       <c r="C325" s="258" t="s">
         <v>365</v>
@@ -30706,8 +30706,8 @@
       <c r="A326" s="261" t="s">
         <v>366</v>
       </c>
-      <c r="B326" s="261" t="s">
-        <v>366</v>
+      <c r="B326" s="261">
+        <v>422601</v>
       </c>
       <c r="C326" s="258" t="s">
         <v>367</v>
@@ -30726,8 +30726,8 @@
       <c r="A327" s="261" t="s">
         <v>368</v>
       </c>
-      <c r="B327" s="261" t="s">
-        <v>368</v>
+      <c r="B327" s="261">
+        <v>422700</v>
       </c>
       <c r="C327" s="258" t="s">
         <v>369</v>
@@ -30746,8 +30746,8 @@
       <c r="A328" s="261" t="s">
         <v>371</v>
       </c>
-      <c r="B328" s="261" t="s">
-        <v>371</v>
+      <c r="B328" s="261">
+        <v>422701</v>
       </c>
       <c r="C328" s="258" t="s">
         <v>372</v>
@@ -30767,7 +30767,7 @@
         <v>4228</v>
       </c>
       <c r="B329" s="261">
-        <v>4228</v>
+        <v>422800</v>
       </c>
       <c r="C329" s="258" t="s">
         <v>373</v>
@@ -30787,7 +30787,7 @@
         <v>4229</v>
       </c>
       <c r="B330" s="261">
-        <v>4229</v>
+        <v>422900</v>
       </c>
       <c r="C330" s="258" t="s">
         <v>374</v>
@@ -30807,7 +30807,7 @@
         <v>4230</v>
       </c>
       <c r="B331" s="261">
-        <v>4230</v>
+        <v>423000</v>
       </c>
       <c r="C331" s="258" t="s">
         <v>375</v>
@@ -30827,7 +30827,7 @@
         <v>4232</v>
       </c>
       <c r="B332" s="261">
-        <v>4232</v>
+        <v>423200</v>
       </c>
       <c r="C332" s="258" t="s">
         <v>376</v>
@@ -30846,8 +30846,8 @@
       <c r="A333" s="261" t="s">
         <v>377</v>
       </c>
-      <c r="B333" s="261" t="s">
-        <v>377</v>
+      <c r="B333" s="261">
+        <v>423308</v>
       </c>
       <c r="C333" s="258" t="s">
         <v>378</v>
@@ -30866,8 +30866,8 @@
       <c r="A334" s="261" t="s">
         <v>379</v>
       </c>
-      <c r="B334" s="261" t="s">
-        <v>379</v>
+      <c r="B334" s="261">
+        <v>423304</v>
       </c>
       <c r="C334" s="258" t="s">
         <v>380</v>
@@ -30886,8 +30886,8 @@
       <c r="A335" s="261" t="s">
         <v>381</v>
       </c>
-      <c r="B335" s="261" t="s">
-        <v>381</v>
+      <c r="B335" s="261">
+        <v>423309</v>
       </c>
       <c r="C335" s="258" t="s">
         <v>382</v>
@@ -30906,8 +30906,8 @@
       <c r="A336" s="261" t="s">
         <v>383</v>
       </c>
-      <c r="B336" s="261" t="s">
-        <v>383</v>
+      <c r="B336" s="261">
+        <v>423316</v>
       </c>
       <c r="C336" s="258" t="s">
         <v>384</v>
@@ -30926,8 +30926,8 @@
       <c r="A337" s="261" t="s">
         <v>385</v>
       </c>
-      <c r="B337" s="261" t="s">
-        <v>385</v>
+      <c r="B337" s="261">
+        <v>423348</v>
       </c>
       <c r="C337" s="258" t="s">
         <v>386</v>
@@ -30946,8 +30946,8 @@
       <c r="A338" s="261" t="s">
         <v>387</v>
       </c>
-      <c r="B338" s="261" t="s">
-        <v>387</v>
+      <c r="B338" s="261">
+        <v>423404</v>
       </c>
       <c r="C338" s="267" t="s">
         <v>388</v>
@@ -30966,8 +30966,8 @@
       <c r="A339" s="261" t="s">
         <v>389</v>
       </c>
-      <c r="B339" s="261" t="s">
-        <v>389</v>
+      <c r="B339" s="261">
+        <v>423408</v>
       </c>
       <c r="C339" s="258" t="s">
         <v>390</v>
@@ -30986,8 +30986,8 @@
       <c r="A340" s="261" t="s">
         <v>391</v>
       </c>
-      <c r="B340" s="261" t="s">
-        <v>391</v>
+      <c r="B340" s="261">
+        <v>423409</v>
       </c>
       <c r="C340" s="258" t="s">
         <v>392</v>
@@ -31006,8 +31006,8 @@
       <c r="A341" s="261" t="s">
         <v>393</v>
       </c>
-      <c r="B341" s="261" t="s">
-        <v>393</v>
+      <c r="B341" s="261">
+        <v>423416</v>
       </c>
       <c r="C341" s="258" t="s">
         <v>384</v>
@@ -31026,8 +31026,8 @@
       <c r="A342" s="261" t="s">
         <v>394</v>
       </c>
-      <c r="B342" s="261" t="s">
-        <v>394</v>
+      <c r="B342" s="261">
+        <v>423448</v>
       </c>
       <c r="C342" s="258" t="s">
         <v>386</v>
@@ -31046,8 +31046,8 @@
       <c r="A343" s="261" t="s">
         <v>395</v>
       </c>
-      <c r="B343" s="261" t="s">
-        <v>395</v>
+      <c r="B343" s="261">
+        <v>423500</v>
       </c>
       <c r="C343" s="258" t="s">
         <v>396</v>
@@ -31066,8 +31066,8 @@
       <c r="A344" s="261" t="s">
         <v>397</v>
       </c>
-      <c r="B344" s="261" t="s">
-        <v>397</v>
+      <c r="B344" s="261">
+        <v>423501</v>
       </c>
       <c r="C344" s="258" t="s">
         <v>398</v>
@@ -31086,8 +31086,8 @@
       <c r="A345" s="261" t="s">
         <v>399</v>
       </c>
-      <c r="B345" s="261" t="s">
-        <v>399</v>
+      <c r="B345" s="261">
+        <v>423600</v>
       </c>
       <c r="C345" s="258" t="s">
         <v>400</v>
@@ -31106,8 +31106,8 @@
       <c r="A346" s="261" t="s">
         <v>401</v>
       </c>
-      <c r="B346" s="261" t="s">
-        <v>401</v>
+      <c r="B346" s="261">
+        <v>423800</v>
       </c>
       <c r="C346" s="258" t="s">
         <v>402</v>
@@ -31126,8 +31126,8 @@
       <c r="A347" s="261" t="s">
         <v>403</v>
       </c>
-      <c r="B347" s="261" t="s">
-        <v>403</v>
+      <c r="B347" s="261">
+        <v>423900</v>
       </c>
       <c r="C347" s="258" t="s">
         <v>404</v>
@@ -31146,8 +31146,8 @@
       <c r="A348" s="261" t="s">
         <v>405</v>
       </c>
-      <c r="B348" s="261" t="s">
-        <v>405</v>
+      <c r="B348" s="261">
+        <v>424000</v>
       </c>
       <c r="C348" s="258" t="s">
         <v>406</v>
@@ -31166,8 +31166,8 @@
       <c r="A349" s="261" t="s">
         <v>407</v>
       </c>
-      <c r="B349" s="261" t="s">
-        <v>407</v>
+      <c r="B349" s="261">
+        <v>424200</v>
       </c>
       <c r="C349" s="258" t="s">
         <v>408</v>
@@ -31186,8 +31186,8 @@
       <c r="A350" s="261" t="s">
         <v>409</v>
       </c>
-      <c r="B350" s="261" t="s">
-        <v>409</v>
+      <c r="B350" s="261">
+        <v>424300</v>
       </c>
       <c r="C350" s="258" t="s">
         <v>410</v>
@@ -31206,8 +31206,8 @@
       <c r="A351" s="261" t="s">
         <v>411</v>
       </c>
-      <c r="B351" s="261" t="s">
-        <v>411</v>
+      <c r="B351" s="261">
+        <v>424301</v>
       </c>
       <c r="C351" s="258" t="s">
         <v>412</v>
@@ -31226,8 +31226,8 @@
       <c r="A352" s="261" t="s">
         <v>413</v>
       </c>
-      <c r="B352" s="261" t="s">
-        <v>413</v>
+      <c r="B352" s="261">
+        <v>424400</v>
       </c>
       <c r="C352" s="258" t="s">
         <v>414</v>
@@ -31246,8 +31246,8 @@
       <c r="A353" s="261" t="s">
         <v>415</v>
       </c>
-      <c r="B353" s="261" t="s">
-        <v>415</v>
+      <c r="B353" s="261">
+        <v>424500</v>
       </c>
       <c r="C353" s="258" t="s">
         <v>416</v>
@@ -31266,8 +31266,8 @@
       <c r="A354" s="261" t="s">
         <v>417</v>
       </c>
-      <c r="B354" s="261" t="s">
-        <v>417</v>
+      <c r="B354" s="261">
+        <v>424600</v>
       </c>
       <c r="C354" s="258" t="s">
         <v>418</v>
@@ -31286,8 +31286,8 @@
       <c r="A355" s="261" t="s">
         <v>419</v>
       </c>
-      <c r="B355" s="261" t="s">
-        <v>419</v>
+      <c r="B355" s="261">
+        <v>424700</v>
       </c>
       <c r="C355" s="258" t="s">
         <v>420</v>
@@ -31306,8 +31306,8 @@
       <c r="A356" s="261" t="s">
         <v>421</v>
       </c>
-      <c r="B356" s="261" t="s">
-        <v>421</v>
+      <c r="B356" s="261">
+        <v>424800</v>
       </c>
       <c r="C356" s="258" t="s">
         <v>422</v>
@@ -31326,8 +31326,8 @@
       <c r="A357" s="261" t="s">
         <v>423</v>
       </c>
-      <c r="B357" s="261" t="s">
-        <v>423</v>
+      <c r="B357" s="261">
+        <v>424801</v>
       </c>
       <c r="C357" s="258" t="s">
         <v>424</v>
@@ -31346,8 +31346,8 @@
       <c r="A358" s="261" t="s">
         <v>425</v>
       </c>
-      <c r="B358" s="261" t="s">
-        <v>425</v>
+      <c r="B358" s="261">
+        <v>424900</v>
       </c>
       <c r="C358" s="258" t="s">
         <v>426</v>
@@ -31366,8 +31366,8 @@
       <c r="A359" s="261" t="s">
         <v>427</v>
       </c>
-      <c r="B359" s="261" t="s">
-        <v>427</v>
+      <c r="B359" s="261">
+        <v>424960</v>
       </c>
       <c r="C359" s="258" t="s">
         <v>428</v>
@@ -31386,8 +31386,8 @@
       <c r="A360" s="261" t="s">
         <v>429</v>
       </c>
-      <c r="B360" s="261" t="s">
-        <v>429</v>
+      <c r="B360" s="261">
+        <v>425000</v>
       </c>
       <c r="C360" s="258" t="s">
         <v>306</v>
@@ -31406,8 +31406,8 @@
       <c r="A361" s="261" t="s">
         <v>430</v>
       </c>
-      <c r="B361" s="261" t="s">
-        <v>430</v>
+      <c r="B361" s="261">
+        <v>425160</v>
       </c>
       <c r="C361" s="258" t="s">
         <v>431</v>
@@ -31427,7 +31427,7 @@
         <v>4256</v>
       </c>
       <c r="B362" s="261">
-        <v>4256</v>
+        <v>425600</v>
       </c>
       <c r="C362" s="258" t="s">
         <v>432</v>
@@ -31446,8 +31446,8 @@
       <c r="A363" s="261" t="s">
         <v>433</v>
       </c>
-      <c r="B363" s="261" t="s">
-        <v>433</v>
+      <c r="B363" s="261">
+        <v>425704</v>
       </c>
       <c r="C363" s="258" t="s">
         <v>434</v>
@@ -31466,8 +31466,8 @@
       <c r="A364" s="261" t="s">
         <v>435</v>
       </c>
-      <c r="B364" s="261" t="s">
-        <v>435</v>
+      <c r="B364" s="261">
+        <v>425708</v>
       </c>
       <c r="C364" s="258" t="s">
         <v>436</v>
@@ -31486,8 +31486,8 @@
       <c r="A365" s="261" t="s">
         <v>437</v>
       </c>
-      <c r="B365" s="261" t="s">
-        <v>437</v>
+      <c r="B365" s="261">
+        <v>425709</v>
       </c>
       <c r="C365" s="258" t="s">
         <v>438</v>
@@ -31506,8 +31506,8 @@
       <c r="A366" s="261" t="s">
         <v>439</v>
       </c>
-      <c r="B366" s="261" t="s">
-        <v>439</v>
+      <c r="B366" s="261">
+        <v>425716</v>
       </c>
       <c r="C366" s="258" t="s">
         <v>440</v>
@@ -31526,8 +31526,8 @@
       <c r="A367" s="261" t="s">
         <v>441</v>
       </c>
-      <c r="B367" s="261" t="s">
-        <v>441</v>
+      <c r="B367" s="261">
+        <v>425748</v>
       </c>
       <c r="C367" s="258" t="s">
         <v>442</v>
@@ -31546,8 +31546,8 @@
       <c r="A368" s="261" t="s">
         <v>443</v>
       </c>
-      <c r="B368" s="261" t="s">
-        <v>443</v>
+      <c r="B368" s="261">
+        <v>420502</v>
       </c>
       <c r="C368" s="258" t="s">
         <v>444</v>
@@ -31566,8 +31566,8 @@
       <c r="A369" s="261" t="s">
         <v>445</v>
       </c>
-      <c r="B369" s="261" t="s">
-        <v>445</v>
+      <c r="B369" s="261">
+        <v>420700</v>
       </c>
       <c r="C369" s="258" t="s">
         <v>446</v>
@@ -32950,7 +32950,7 @@
       <c r="A436" s="294">
         <v>11111111</v>
       </c>
-      <c r="B436" s="357" t="str">
+      <c r="B436" s="357">
         <f>MID(A436,2,6)</f>
         <v>111111</v>
       </c>
@@ -32961,7 +32961,7 @@
     <row r="437" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A437" s="272"/>
       <c r="B437" s="362">
-        <v>4401</v>
+        <v>440100</v>
       </c>
       <c r="C437" s="367"/>
       <c r="D437" s="358" t="s">
@@ -32974,7 +32974,7 @@
     </row>
     <row r="438" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B438" s="381">
-        <v>4402</v>
+        <v>440200</v>
       </c>
       <c r="C438" s="389" t="s">
         <v>522</v>
@@ -32991,7 +32991,7 @@
     </row>
     <row r="439" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B439" s="362">
-        <v>4403</v>
+        <v>440300</v>
       </c>
       <c r="C439" s="367"/>
       <c r="D439" s="358" t="s">
@@ -33004,7 +33004,7 @@
     </row>
     <row r="440" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B440" s="362">
-        <v>4404</v>
+        <v>440400</v>
       </c>
       <c r="C440" s="367"/>
       <c r="D440" s="358" t="s">
@@ -33017,7 +33017,7 @@
     </row>
     <row r="441" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B441" s="362">
-        <v>4405</v>
+        <v>440500</v>
       </c>
       <c r="C441" s="367"/>
       <c r="D441" s="358" t="s">
@@ -33030,7 +33030,7 @@
     </row>
     <row r="442" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B442" s="362">
-        <v>4406</v>
+        <v>440600</v>
       </c>
       <c r="C442" s="367" t="s">
         <v>524</v>
@@ -33047,7 +33047,7 @@
     </row>
     <row r="443" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B443" s="397">
-        <v>4407</v>
+        <v>440700</v>
       </c>
       <c r="C443" s="382" t="s">
         <v>525</v>
@@ -33064,7 +33064,7 @@
     </row>
     <row r="444" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B444" s="362">
-        <v>4408</v>
+        <v>440800</v>
       </c>
       <c r="C444" s="171"/>
       <c r="D444" s="358" t="s">
@@ -33077,7 +33077,7 @@
     </row>
     <row r="445" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B445" s="362">
-        <v>4409</v>
+        <v>440900</v>
       </c>
       <c r="C445" s="171"/>
       <c r="D445" s="358" t="s">
@@ -33090,7 +33090,7 @@
     </row>
     <row r="446" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B446" s="362">
-        <v>4410</v>
+        <v>441000</v>
       </c>
       <c r="C446" s="171"/>
       <c r="D446" s="358" t="s">
@@ -33103,7 +33103,7 @@
     </row>
     <row r="447" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B447" s="362">
-        <v>4411</v>
+        <v>441100</v>
       </c>
       <c r="C447" s="171"/>
       <c r="D447" s="358" t="s">
@@ -33116,7 +33116,7 @@
     </row>
     <row r="448" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B448" s="397">
-        <v>4412</v>
+        <v>441200</v>
       </c>
       <c r="C448" s="382" t="s">
         <v>526</v>
@@ -33133,7 +33133,7 @@
     </row>
     <row r="449" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B449" s="381">
-        <v>4413</v>
+        <v>441300</v>
       </c>
       <c r="C449" s="382" t="s">
         <v>528</v>
@@ -33149,8 +33149,8 @@
       </c>
     </row>
     <row r="450" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B450" s="381" t="s">
-        <v>2219</v>
+      <c r="B450" s="381">
+        <v>441400</v>
       </c>
       <c r="C450" s="382" t="s">
         <v>529</v>
@@ -33166,8 +33166,8 @@
       </c>
     </row>
     <row r="451" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B451" s="381" t="s">
-        <v>530</v>
+      <c r="B451" s="381">
+        <v>441401</v>
       </c>
       <c r="C451" s="382" t="s">
         <v>531</v>
@@ -33183,8 +33183,8 @@
       </c>
     </row>
     <row r="452" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B452" s="362" t="s">
-        <v>2214</v>
+      <c r="B452" s="362">
+        <v>441500</v>
       </c>
       <c r="C452" s="171" t="s">
         <v>2212</v>
@@ -33196,8 +33196,8 @@
       </c>
     </row>
     <row r="453" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B453" s="362" t="s">
-        <v>2213</v>
+      <c r="B453" s="362">
+        <v>441501</v>
       </c>
       <c r="C453" s="171" t="s">
         <v>2211</v>
@@ -33210,7 +33210,7 @@
     </row>
     <row r="454" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B454" s="397">
-        <v>4416</v>
+        <v>441600</v>
       </c>
       <c r="C454" s="382" t="s">
         <v>532</v>
@@ -33261,7 +33261,7 @@
     </row>
     <row r="457" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B457" s="397">
-        <v>4418</v>
+        <v>441800</v>
       </c>
       <c r="C457" s="382" t="s">
         <v>534</v>
@@ -33277,8 +33277,8 @@
       </c>
     </row>
     <row r="458" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B458" s="397" t="s">
-        <v>535</v>
+      <c r="B458" s="397">
+        <v>441900</v>
       </c>
       <c r="C458" s="382" t="s">
         <v>536</v>
@@ -33294,8 +33294,8 @@
       </c>
     </row>
     <row r="459" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B459" s="397" t="s">
-        <v>537</v>
+      <c r="B459" s="397">
+        <v>441901</v>
       </c>
       <c r="C459" s="382" t="s">
         <v>538</v>
@@ -33312,7 +33312,7 @@
     </row>
     <row r="460" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B460" s="362">
-        <v>4420</v>
+        <v>442000</v>
       </c>
       <c r="C460" s="378" t="s">
         <v>539</v>
@@ -33327,7 +33327,7 @@
     </row>
     <row r="461" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B461" s="381">
-        <v>4421</v>
+        <v>442100</v>
       </c>
       <c r="C461" s="382" t="s">
         <v>540</v>
@@ -33343,8 +33343,8 @@
       </c>
     </row>
     <row r="462" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B462" s="381" t="s">
-        <v>541</v>
+      <c r="B462" s="381">
+        <v>442200</v>
       </c>
       <c r="C462" s="382" t="s">
         <v>542</v>
@@ -33360,8 +33360,8 @@
       </c>
     </row>
     <row r="463" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B463" s="381" t="s">
-        <v>544</v>
+      <c r="B463" s="381">
+        <v>442204</v>
       </c>
       <c r="C463" s="382" t="s">
         <v>545</v>
@@ -33377,8 +33377,8 @@
       </c>
     </row>
     <row r="464" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B464" s="381" t="s">
-        <v>546</v>
+      <c r="B464" s="381">
+        <v>442206</v>
       </c>
       <c r="C464" s="382" t="s">
         <v>547</v>
@@ -33394,8 +33394,8 @@
       </c>
     </row>
     <row r="465" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B465" s="381" t="s">
-        <v>548</v>
+      <c r="B465" s="381">
+        <v>442238</v>
       </c>
       <c r="C465" s="382" t="s">
         <v>549</v>
@@ -33412,7 +33412,7 @@
     </row>
     <row r="466" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B466" s="362">
-        <v>4423</v>
+        <v>442300</v>
       </c>
       <c r="C466" s="171"/>
       <c r="D466" s="358" t="s">
@@ -33425,7 +33425,7 @@
     </row>
     <row r="467" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B467" s="362">
-        <v>4424</v>
+        <v>442400</v>
       </c>
       <c r="C467" s="171"/>
       <c r="D467" s="358" t="s">
@@ -33438,7 +33438,7 @@
     </row>
     <row r="468" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B468" s="362">
-        <v>4425</v>
+        <v>442500</v>
       </c>
       <c r="C468" s="171"/>
       <c r="D468" s="358" t="s">
@@ -33450,8 +33450,8 @@
       <c r="F468" s="29"/>
     </row>
     <row r="469" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B469" s="381" t="s">
-        <v>2216</v>
+      <c r="B469" s="381">
+        <v>442600</v>
       </c>
       <c r="C469" s="393" t="s">
         <v>551</v>
@@ -33467,8 +33467,8 @@
       </c>
     </row>
     <row r="470" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B470" s="381" t="s">
-        <v>2217</v>
+      <c r="B470" s="381">
+        <v>442601</v>
       </c>
       <c r="C470" s="393" t="s">
         <v>2218</v>
@@ -33485,7 +33485,7 @@
     </row>
     <row r="471" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B471" s="362">
-        <v>4427</v>
+        <v>442700</v>
       </c>
       <c r="C471" s="171"/>
       <c r="D471" s="358" t="s">
@@ -33498,7 +33498,7 @@
     </row>
     <row r="472" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B472" s="362">
-        <v>4428</v>
+        <v>442800</v>
       </c>
       <c r="C472" s="171"/>
       <c r="D472" s="358" t="s">
@@ -33510,8 +33510,8 @@
       <c r="F472" s="29"/>
     </row>
     <row r="473" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B473" s="362" t="s">
-        <v>2193</v>
+      <c r="B473" s="362">
+        <v>442909</v>
       </c>
       <c r="C473" s="171" t="s">
         <v>2194</v>
@@ -33527,8 +33527,8 @@
       </c>
     </row>
     <row r="474" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B474" s="362" t="s">
-        <v>2195</v>
+      <c r="B474" s="362">
+        <v>442904</v>
       </c>
       <c r="C474" s="171" t="s">
         <v>2196</v>
@@ -33544,8 +33544,8 @@
       </c>
     </row>
     <row r="475" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B475" s="362" t="s">
-        <v>2197</v>
+      <c r="B475" s="362">
+        <v>442906</v>
       </c>
       <c r="C475" s="171" t="s">
         <v>2198</v>
@@ -33561,8 +33561,8 @@
       </c>
     </row>
     <row r="476" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B476" s="362" t="s">
-        <v>2199</v>
+      <c r="B476" s="362">
+        <v>442924</v>
       </c>
       <c r="C476" s="171" t="s">
         <v>2200</v>
@@ -33578,8 +33578,8 @@
       </c>
     </row>
     <row r="477" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B477" s="362" t="s">
-        <v>2201</v>
+      <c r="B477" s="362">
+        <v>442938</v>
       </c>
       <c r="C477" s="171" t="s">
         <v>2202</v>
@@ -33603,7 +33603,7 @@
     </row>
     <row r="479" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B479" s="397">
-        <v>4430</v>
+        <v>443000</v>
       </c>
       <c r="C479" s="171" t="s">
         <v>552</v>
@@ -33619,8 +33619,8 @@
       </c>
     </row>
     <row r="480" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B480" s="397" t="s">
-        <v>553</v>
+      <c r="B480" s="397">
+        <v>443100</v>
       </c>
       <c r="C480" s="382" t="s">
         <v>554</v>
@@ -33636,8 +33636,8 @@
       </c>
     </row>
     <row r="481" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B481" s="397" t="s">
-        <v>555</v>
+      <c r="B481" s="397">
+        <v>443101</v>
       </c>
       <c r="C481" s="386" t="s">
         <v>556</v>
@@ -33654,7 +33654,7 @@
     </row>
     <row r="482" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B482" s="381">
-        <v>4432</v>
+        <v>443200</v>
       </c>
       <c r="C482" s="382" t="s">
         <v>557</v>
@@ -33671,7 +33671,7 @@
     </row>
     <row r="483" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B483" s="362">
-        <v>4433</v>
+        <v>443300</v>
       </c>
       <c r="C483" s="171" t="s">
         <v>558</v>
@@ -33689,7 +33689,7 @@
         <v>559</v>
       </c>
       <c r="B484" s="397">
-        <v>4434</v>
+        <v>443400</v>
       </c>
       <c r="C484" s="386" t="s">
         <v>560</v>
@@ -33706,7 +33706,7 @@
     </row>
     <row r="485" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B485" s="381">
-        <v>4435</v>
+        <v>443500</v>
       </c>
       <c r="C485" s="393" t="s">
         <v>561</v>
@@ -33723,7 +33723,7 @@
     </row>
     <row r="486" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B486" s="362">
-        <v>4436</v>
+        <v>443600</v>
       </c>
       <c r="C486" s="171"/>
       <c r="D486" s="358" t="s">
@@ -33736,7 +33736,7 @@
     </row>
     <row r="487" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B487" s="362">
-        <v>4437</v>
+        <v>443700</v>
       </c>
       <c r="C487" s="171" t="s">
         <v>562</v>
@@ -33751,7 +33751,7 @@
     </row>
     <row r="488" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B488" s="362">
-        <v>4438</v>
+        <v>443800</v>
       </c>
       <c r="C488" s="171" t="s">
         <v>2215</v>
@@ -33763,8 +33763,8 @@
       </c>
     </row>
     <row r="489" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B489" s="362" t="s">
-        <v>563</v>
+      <c r="B489" s="362">
+        <v>443900</v>
       </c>
       <c r="C489" s="171" t="s">
         <v>564</v>
@@ -33782,7 +33782,7 @@
     </row>
     <row r="490" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B490" s="381">
-        <v>4440</v>
+        <v>444000</v>
       </c>
       <c r="C490" s="382" t="s">
         <v>565</v>
@@ -33799,7 +33799,7 @@
     </row>
     <row r="491" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B491" s="397">
-        <v>4441</v>
+        <v>444100</v>
       </c>
       <c r="C491" s="394" t="s">
         <v>566</v>
@@ -33816,7 +33816,7 @@
     </row>
     <row r="492" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B492" s="381">
-        <v>4442</v>
+        <v>444200</v>
       </c>
       <c r="C492" s="382" t="s">
         <v>567</v>
@@ -33833,7 +33833,7 @@
     </row>
     <row r="493" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B493" s="381">
-        <v>4443</v>
+        <v>444300</v>
       </c>
       <c r="C493" s="382" t="s">
         <v>569</v>
@@ -33850,7 +33850,7 @@
     </row>
     <row r="494" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B494" s="381">
-        <v>4444</v>
+        <v>444400</v>
       </c>
       <c r="C494" s="382" t="s">
         <v>570</v>
@@ -33867,7 +33867,7 @@
     </row>
     <row r="495" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B495" s="362">
-        <v>4445</v>
+        <v>444500</v>
       </c>
       <c r="C495" s="171"/>
       <c r="D495" s="358" t="s">
@@ -33880,7 +33880,7 @@
     </row>
     <row r="496" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B496" s="362">
-        <v>4446</v>
+        <v>444600</v>
       </c>
       <c r="C496" s="171"/>
       <c r="D496" s="358" t="s">
@@ -33893,7 +33893,7 @@
     </row>
     <row r="497" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B497" s="362">
-        <v>4447</v>
+        <v>444700</v>
       </c>
       <c r="C497" s="171"/>
       <c r="D497" s="358" t="s">
@@ -33906,7 +33906,7 @@
     </row>
     <row r="498" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B498" s="381">
-        <v>4448</v>
+        <v>444800</v>
       </c>
       <c r="C498" s="382" t="s">
         <v>571</v>
@@ -33922,8 +33922,8 @@
       </c>
     </row>
     <row r="499" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B499" s="362" t="s">
-        <v>572</v>
+      <c r="B499" s="362">
+        <v>444890</v>
       </c>
       <c r="C499" s="378" t="s">
         <v>573</v>
@@ -33936,7 +33936,7 @@
     </row>
     <row r="500" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B500" s="362">
-        <v>4449</v>
+        <v>444900</v>
       </c>
       <c r="C500" s="171"/>
       <c r="D500" s="358" t="s">
@@ -33949,7 +33949,7 @@
     </row>
     <row r="501" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B501" s="362">
-        <v>4450</v>
+        <v>445000</v>
       </c>
       <c r="C501" s="171"/>
       <c r="D501" s="358" t="s">
@@ -33962,7 +33962,7 @@
     </row>
     <row r="502" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B502" s="362">
-        <v>4451</v>
+        <v>445100</v>
       </c>
       <c r="C502" s="171"/>
       <c r="D502" s="361" t="s">
@@ -33975,7 +33975,7 @@
     </row>
     <row r="503" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B503" s="362">
-        <v>4452</v>
+        <v>445200</v>
       </c>
       <c r="C503" s="171"/>
       <c r="D503" s="358" t="s">
@@ -33988,7 +33988,7 @@
     </row>
     <row r="504" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B504" s="381">
-        <v>4453</v>
+        <v>445300</v>
       </c>
       <c r="C504" s="382" t="s">
         <v>574</v>
@@ -34006,7 +34006,7 @@
     </row>
     <row r="505" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B505" s="397">
-        <v>4454</v>
+        <v>445400</v>
       </c>
       <c r="C505" s="382" t="s">
         <v>576</v>
@@ -34026,7 +34026,7 @@
         <v>2188</v>
       </c>
       <c r="B506" s="397">
-        <v>4455</v>
+        <v>445500</v>
       </c>
       <c r="C506" s="382" t="s">
         <v>577</v>
@@ -34045,8 +34045,8 @@
       <c r="A507" s="221" t="s">
         <v>211</v>
       </c>
-      <c r="B507" s="381" t="s">
-        <v>2220</v>
+      <c r="B507" s="381">
+        <v>445660</v>
       </c>
       <c r="C507" s="386" t="s">
         <v>2222</v>
@@ -34062,8 +34062,8 @@
       </c>
     </row>
     <row r="508" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B508" s="381" t="s">
-        <v>2221</v>
+      <c r="B508" s="381">
+        <v>445600</v>
       </c>
       <c r="C508" s="386" t="s">
         <v>2222</v>
@@ -34079,8 +34079,8 @@
       </c>
     </row>
     <row r="509" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B509" s="381" t="s">
-        <v>578</v>
+      <c r="B509" s="381">
+        <v>445700</v>
       </c>
       <c r="C509" s="382" t="s">
         <v>579</v>
@@ -34096,8 +34096,8 @@
       </c>
     </row>
     <row r="510" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B510" s="381" t="s">
-        <v>580</v>
+      <c r="B510" s="381">
+        <v>445738</v>
       </c>
       <c r="C510" s="382" t="s">
         <v>581</v>
@@ -34113,8 +34113,8 @@
       </c>
     </row>
     <row r="511" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B511" s="381" t="s">
-        <v>582</v>
+      <c r="B511" s="381">
+        <v>445706</v>
       </c>
       <c r="C511" s="382" t="s">
         <v>583</v>
@@ -34130,8 +34130,8 @@
       </c>
     </row>
     <row r="512" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B512" s="381" t="s">
-        <v>584</v>
+      <c r="B512" s="381">
+        <v>445704</v>
       </c>
       <c r="C512" s="382" t="s">
         <v>585</v>
@@ -34147,8 +34147,8 @@
       </c>
     </row>
     <row r="513" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B513" s="381" t="s">
-        <v>2203</v>
+      <c r="B513" s="381">
+        <v>445724</v>
       </c>
       <c r="C513" s="382" t="s">
         <v>2204</v>
@@ -34165,7 +34165,7 @@
     </row>
     <row r="514" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B514" s="381">
-        <v>4458</v>
+        <v>445800</v>
       </c>
       <c r="C514" s="382" t="s">
         <v>586</v>
@@ -34196,7 +34196,7 @@
     </row>
     <row r="517" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B517" s="362">
-        <v>4458</v>
+        <v>445800</v>
       </c>
       <c r="C517" s="171" t="s">
         <v>588</v>
@@ -34213,7 +34213,7 @@
     </row>
     <row r="518" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B518" s="381">
-        <v>4459</v>
+        <v>445900</v>
       </c>
       <c r="C518" s="382" t="s">
         <v>589</v>
@@ -34230,7 +34230,7 @@
     </row>
     <row r="519" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B519" s="362">
-        <v>4460</v>
+        <v>446000</v>
       </c>
       <c r="C519" s="171" t="s">
         <v>591</v>
@@ -34247,7 +34247,7 @@
     </row>
     <row r="520" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B520" s="362">
-        <v>4461</v>
+        <v>446100</v>
       </c>
       <c r="C520" s="171"/>
       <c r="D520" s="358" t="s">
@@ -34260,7 +34260,7 @@
     </row>
     <row r="521" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B521" s="362">
-        <v>4462</v>
+        <v>446200</v>
       </c>
       <c r="C521" s="171"/>
       <c r="D521" s="358" t="s">
@@ -34273,7 +34273,7 @@
     </row>
     <row r="522" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B522" s="362">
-        <v>4463</v>
+        <v>446300</v>
       </c>
       <c r="C522" s="171"/>
       <c r="D522" s="358" t="s">
@@ -34286,7 +34286,7 @@
     </row>
     <row r="523" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B523" s="362">
-        <v>4464</v>
+        <v>446400</v>
       </c>
       <c r="C523" s="171"/>
       <c r="D523" s="358" t="s">
@@ -34299,7 +34299,7 @@
     </row>
     <row r="524" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B524" s="362">
-        <v>4465</v>
+        <v>446500</v>
       </c>
       <c r="C524" s="171"/>
       <c r="D524" s="358" t="s">
@@ -34312,7 +34312,7 @@
     </row>
     <row r="525" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B525" s="362">
-        <v>4466</v>
+        <v>446600</v>
       </c>
       <c r="C525" s="171"/>
       <c r="D525" s="358" t="s">
@@ -34325,7 +34325,7 @@
     </row>
     <row r="526" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B526" s="362">
-        <v>4467</v>
+        <v>446700</v>
       </c>
       <c r="C526" s="171"/>
       <c r="D526" s="358" t="s">
@@ -34338,7 +34338,7 @@
     </row>
     <row r="527" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B527" s="397">
-        <v>4468</v>
+        <v>446800</v>
       </c>
       <c r="C527" s="382" t="s">
         <v>593</v>
@@ -34355,7 +34355,7 @@
     </row>
     <row r="528" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B528" s="362">
-        <v>4469</v>
+        <v>446900</v>
       </c>
       <c r="C528" s="171"/>
       <c r="D528" s="358" t="s">
@@ -34370,7 +34370,7 @@
     </row>
     <row r="529" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B529" s="362">
-        <v>4470</v>
+        <v>447000</v>
       </c>
       <c r="C529" s="171"/>
       <c r="D529" s="358" t="s">
@@ -34385,7 +34385,7 @@
     </row>
     <row r="530" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B530" s="397">
-        <v>4471</v>
+        <v>447100</v>
       </c>
       <c r="C530" s="382" t="s">
         <v>596</v>
@@ -34401,8 +34401,8 @@
       </c>
     </row>
     <row r="531" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B531" s="397" t="s">
-        <v>597</v>
+      <c r="B531" s="397">
+        <v>447200</v>
       </c>
       <c r="C531" s="386" t="s">
         <v>598</v>
@@ -34418,8 +34418,8 @@
       </c>
     </row>
     <row r="532" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B532" s="397" t="s">
-        <v>599</v>
+      <c r="B532" s="397">
+        <v>447201</v>
       </c>
       <c r="C532" s="386" t="s">
         <v>600</v>
@@ -34439,7 +34439,7 @@
         <v>601</v>
       </c>
       <c r="B533" s="397">
-        <v>4473</v>
+        <v>447300</v>
       </c>
       <c r="C533" s="382" t="s">
         <v>602</v>
@@ -34456,7 +34456,7 @@
     </row>
     <row r="534" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B534" s="362">
-        <v>4474</v>
+        <v>447400</v>
       </c>
       <c r="C534" s="171"/>
       <c r="D534" s="363" t="s">
@@ -34469,7 +34469,7 @@
     </row>
     <row r="535" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B535" s="362">
-        <v>4475</v>
+        <v>447500</v>
       </c>
       <c r="C535" s="171"/>
       <c r="D535" s="362"/>
@@ -34481,7 +34481,7 @@
         <v>2186</v>
       </c>
       <c r="B536" s="397">
-        <v>4476</v>
+        <v>447600</v>
       </c>
       <c r="C536" s="171" t="s">
         <v>2180</v>
@@ -34498,7 +34498,7 @@
     </row>
     <row r="537" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B537" s="380">
-        <v>4477</v>
+        <v>447700</v>
       </c>
       <c r="C537" s="171"/>
       <c r="D537" s="170"/>
@@ -34507,7 +34507,7 @@
     </row>
     <row r="538" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B538" s="380">
-        <v>4478</v>
+        <v>447800</v>
       </c>
       <c r="C538" s="171"/>
       <c r="D538" s="170"/>
@@ -34516,7 +34516,7 @@
     </row>
     <row r="539" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B539" s="362">
-        <v>4479</v>
+        <v>447900</v>
       </c>
       <c r="C539" s="171"/>
       <c r="D539" s="170"/>
@@ -34525,7 +34525,7 @@
     </row>
     <row r="540" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B540" s="396">
-        <v>4480</v>
+        <v>448000</v>
       </c>
       <c r="C540" s="395" t="s">
         <v>2191</v>
@@ -34542,7 +34542,7 @@
     </row>
     <row r="541" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B541" s="380">
-        <v>4481</v>
+        <v>448100</v>
       </c>
       <c r="C541" s="171"/>
       <c r="D541" s="170"/>
@@ -34554,7 +34554,7 @@
         <v>4236</v>
       </c>
       <c r="B542" s="397">
-        <v>4482</v>
+        <v>448200</v>
       </c>
       <c r="C542" s="171" t="s">
         <v>2189</v>
@@ -34571,7 +34571,7 @@
     </row>
     <row r="543" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B543" s="380">
-        <v>4483</v>
+        <v>448300</v>
       </c>
       <c r="C543" s="171"/>
       <c r="D543" s="170"/>
@@ -34583,7 +34583,7 @@
         <v>4301</v>
       </c>
       <c r="B544" s="396">
-        <v>4484</v>
+        <v>448400</v>
       </c>
       <c r="C544" s="171" t="s">
         <v>2182</v>
@@ -34603,7 +34603,7 @@
         <v>4314</v>
       </c>
       <c r="B545" s="397">
-        <v>4485</v>
+        <v>448500</v>
       </c>
       <c r="C545" s="171" t="s">
         <v>2181</v>
@@ -34620,7 +34620,7 @@
     </row>
     <row r="546" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B546" s="396">
-        <v>4486</v>
+        <v>448600</v>
       </c>
       <c r="C546" s="171" t="s">
         <v>2187</v>
@@ -34636,8 +34636,8 @@
       </c>
     </row>
     <row r="547" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B547" s="380" t="s">
-        <v>2183</v>
+      <c r="B547" s="380">
+        <v>448760</v>
       </c>
       <c r="C547" s="171" t="s">
         <v>2185</v>
@@ -34654,7 +34654,7 @@
     </row>
     <row r="548" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B548" s="380">
-        <v>4487</v>
+        <v>448700</v>
       </c>
       <c r="C548" s="171" t="s">
         <v>2184</v>
@@ -34671,7 +34671,7 @@
     </row>
     <row r="549" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B549" s="362">
-        <v>4488</v>
+        <v>448800</v>
       </c>
       <c r="C549" s="171" t="s">
         <v>605</v>
@@ -34688,7 +34688,7 @@
     </row>
     <row r="550" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B550" s="396">
-        <v>4489</v>
+        <v>448900</v>
       </c>
       <c r="C550" s="382" t="s">
         <v>606</v>
@@ -34705,7 +34705,7 @@
     </row>
     <row r="551" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B551" s="380">
-        <v>4490</v>
+        <v>449000</v>
       </c>
       <c r="C551" s="171"/>
       <c r="D551" s="170"/>
@@ -34714,7 +34714,7 @@
     </row>
     <row r="552" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B552" s="362">
-        <v>4491</v>
+        <v>449100</v>
       </c>
       <c r="C552" s="171"/>
       <c r="D552" s="170"/>
@@ -34722,8 +34722,8 @@
       <c r="F552" s="29"/>
     </row>
     <row r="553" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B553" s="396" t="s">
-        <v>607</v>
+      <c r="B553" s="396">
+        <v>449200</v>
       </c>
       <c r="C553" s="171" t="s">
         <v>608</v>
@@ -34739,8 +34739,8 @@
       </c>
     </row>
     <row r="554" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B554" s="380" t="s">
-        <v>609</v>
+      <c r="B554" s="380">
+        <v>449290</v>
       </c>
       <c r="C554" s="171" t="s">
         <v>610</v>
@@ -34756,8 +34756,8 @@
       </c>
     </row>
     <row r="555" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B555" s="380" t="s">
-        <v>2209</v>
+      <c r="B555" s="380">
+        <v>449301</v>
       </c>
       <c r="C555" s="171" t="s">
         <v>2210</v>
@@ -34773,8 +34773,8 @@
       </c>
     </row>
     <row r="556" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B556" s="397" t="s">
-        <v>611</v>
+      <c r="B556" s="397">
+        <v>449404</v>
       </c>
       <c r="C556" s="171" t="s">
         <v>2205</v>
@@ -34790,8 +34790,8 @@
       </c>
     </row>
     <row r="557" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B557" s="362" t="s">
-        <v>612</v>
+      <c r="B557" s="362">
+        <v>449406</v>
       </c>
       <c r="C557" s="171" t="s">
         <v>2206</v>
@@ -34807,8 +34807,8 @@
       </c>
     </row>
     <row r="558" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B558" s="362" t="s">
-        <v>613</v>
+      <c r="B558" s="362">
+        <v>449409</v>
       </c>
       <c r="C558" s="171" t="s">
         <v>2207</v>
@@ -34824,8 +34824,8 @@
       </c>
     </row>
     <row r="559" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B559" s="362" t="s">
-        <v>614</v>
+      <c r="B559" s="362">
+        <v>449424</v>
       </c>
       <c r="C559" s="171" t="s">
         <v>2208</v>
@@ -34855,8 +34855,8 @@
       <c r="F561" s="29"/>
     </row>
     <row r="562" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B562" s="380" t="s">
-        <v>615</v>
+      <c r="B562" s="380">
+        <v>449500</v>
       </c>
       <c r="C562" s="171" t="s">
         <v>616</v>
@@ -34872,8 +34872,8 @@
       </c>
     </row>
     <row r="563" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B563" s="380" t="s">
-        <v>617</v>
+      <c r="B563" s="380">
+        <v>449504</v>
       </c>
       <c r="C563" s="171" t="s">
         <v>618</v>
@@ -34889,8 +34889,8 @@
       </c>
     </row>
     <row r="564" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B564" s="380" t="s">
-        <v>619</v>
+      <c r="B564" s="380">
+        <v>449506</v>
       </c>
       <c r="C564" s="171" t="s">
         <v>620</v>
@@ -34906,8 +34906,8 @@
       </c>
     </row>
     <row r="565" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B565" s="380" t="s">
-        <v>621</v>
+      <c r="B565" s="380">
+        <v>449509</v>
       </c>
       <c r="C565" s="171" t="s">
         <v>622</v>
@@ -34923,8 +34923,8 @@
       </c>
     </row>
     <row r="566" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B566" s="380" t="s">
-        <v>623</v>
+      <c r="B566" s="380">
+        <v>449524</v>
       </c>
       <c r="C566" s="171" t="s">
         <v>624</v>
@@ -34940,8 +34940,8 @@
       </c>
     </row>
     <row r="567" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B567" s="380" t="s">
-        <v>625</v>
+      <c r="B567" s="380">
+        <v>449538</v>
       </c>
       <c r="C567" s="171" t="s">
         <v>626</v>
@@ -34958,7 +34958,7 @@
     </row>
     <row r="568" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B568" s="391">
-        <v>4496</v>
+        <v>449600</v>
       </c>
       <c r="C568" s="382" t="s">
         <v>2192</v>
@@ -34978,7 +34978,7 @@
         <v>4323</v>
       </c>
       <c r="B569" s="397">
-        <v>4497</v>
+        <v>449700</v>
       </c>
       <c r="C569" s="171" t="s">
         <v>2190</v>
@@ -34995,7 +34995,7 @@
     </row>
     <row r="570" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B570" s="380">
-        <v>4498</v>
+        <v>449800</v>
       </c>
       <c r="C570" s="171"/>
       <c r="D570" s="170"/>
@@ -35004,7 +35004,7 @@
     </row>
     <row r="571" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B571" s="295">
-        <v>4499</v>
+        <v>449900</v>
       </c>
       <c r="F571" s="380"/>
     </row>

</xml_diff>

<commit_message>
feat: agregar precios 443102 y 445401 a BD jeans Dama PLANILLA 44
Dos variantes de la Cole 44 tenian precio en la web ($25.990) pero no
en la BD del Excel — el VLOOKUP no los encontraba al descargar pedidos.
Se agregan en filas 572-573 de la hoja BD jeans Dama.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PLANILLA 44 LISTA PRECIO FINAL.xlsx
+++ b/PLANILLA 44 LISTA PRECIO FINAL.xlsx
@@ -35009,10 +35009,40 @@
       <c r="F571" s="380"/>
     </row>
     <row r="572" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="F572" s="380"/>
+      <c r="A572" s="224"/>
+      <c r="B572" s="397">
+        <v>443102</v>
+      </c>
+      <c r="C572" s="382" t="s">
+        <v>556</v>
+      </c>
+      <c r="D572" s="383" t="s">
+        <v>138</v>
+      </c>
+      <c r="E572" s="383" t="s">
+        <v>41</v>
+      </c>
+      <c r="F572" s="384">
+        <v>25990</v>
+      </c>
     </row>
     <row r="573" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="F573" s="380"/>
+      <c r="A573" s="224"/>
+      <c r="B573" s="397">
+        <v>445401</v>
+      </c>
+      <c r="C573" s="382" t="s">
+        <v>576</v>
+      </c>
+      <c r="D573" s="383" t="s">
+        <v>138</v>
+      </c>
+      <c r="E573" s="383" t="s">
+        <v>105</v>
+      </c>
+      <c r="F573" s="384">
+        <v>25990</v>
+      </c>
     </row>
     <row r="574" spans="1:6" x14ac:dyDescent="0.3">
       <c r="F574" s="380"/>

</xml_diff>

<commit_message>
fix: agregar 4440-60 y 4486-01 a BD jeans Dama PLANILLA 44 para evitar #N/D en precio
</commit_message>
<xml_diff>
--- a/PLANILLA 44 LISTA PRECIO FINAL.xlsx
+++ b/PLANILLA 44 LISTA PRECIO FINAL.xlsx
@@ -35045,10 +35045,40 @@
       </c>
     </row>
     <row r="574" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="F574" s="380"/>
+      <c r="A574" s="224"/>
+      <c r="B574" s="397">
+        <v>444060</v>
+      </c>
+      <c r="C574" s="382" t="s">
+        <v>565</v>
+      </c>
+      <c r="D574" s="383" t="s">
+        <v>141</v>
+      </c>
+      <c r="E574" s="383" t="s">
+        <v>186</v>
+      </c>
+      <c r="F574" s="384">
+        <v>25990</v>
+      </c>
     </row>
     <row r="575" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="F575" s="380"/>
+      <c r="A575" s="224"/>
+      <c r="B575" s="397">
+        <v>448601</v>
+      </c>
+      <c r="C575" s="382" t="s">
+        <v>2187</v>
+      </c>
+      <c r="D575" s="383" t="s">
+        <v>141</v>
+      </c>
+      <c r="E575" s="383" t="s">
+        <v>603</v>
+      </c>
+      <c r="F575" s="384">
+        <v>25990</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A437:G477" xr:uid="{00000000-0009-0000-0000-000004000000}"/>

</xml_diff>